<commit_message>
LS recalculado (Moore), origem do CN (ANA BR_CN-2022) e ponto de retomada
- Fator LS refeito por Moore e Burch (1986) sobre o MDE corrigido em UTM;
  scripts, planilhas, mapas e tabelas migrados para o LS novo
- Secao 3.3 do TCC conferida contra os rasters; CN identificado como o
  raster BR_CN-2022 da ANA (notas, secao 25)
- Referencias consolidadas em ordem alfabetica com DOI
- README: secao "Onde estamos agora (17/10/2026)" com pendencias para retomar
- .gitignore: exclui o Plano PCJ completo (188 MB) e arquivos pesados do
  pacote do evento 11 (regeraveis)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Comparacao_Modelos_TCC.xlsx
+++ b/Comparacao_Modelos_TCC.xlsx
@@ -983,31 +983,31 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.1323803145370838</v>
+        <v>0.01021554737345453</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>0.4975114843344086</v>
+        <v>0.5014561479980195</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>0.3746269922765456</v>
+        <v>0.3804165146048779</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>0.8923189156917287</v>
+        <v>0.8926167512266159</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-16.48156760815043</v>
+        <v>-16.14184757409659</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>-13.04561155503808</v>
+        <v>-12.08513115046434</v>
       </c>
       <c r="K10" s="17" t="n">
-        <v>28.47444917497896</v>
+        <v>28.47307387632832</v>
       </c>
       <c r="L10" s="16" t="n">
-        <v>0.07266725235513061</v>
+        <v>0.07702056088139086</v>
       </c>
       <c r="M10" s="16" t="n">
-        <v>0.5613991714495616</v>
+        <v>0.567804501948117</v>
       </c>
       <c r="N10" s="13" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>449.3170466927465</v>
       </c>
       <c r="H4" s="35" t="n">
-        <v>327.9092437431237</v>
+        <v>345.3114725244459</v>
       </c>
       <c r="I4" s="35" t="n">
         <v>325.6612740094749</v>
@@ -1487,7 +1487,7 @@
         <v>1952.709995741231</v>
       </c>
       <c r="H5" s="35" t="n">
-        <v>555.4666538365967</v>
+        <v>556.7738625138491</v>
       </c>
       <c r="I5" s="35" t="n">
         <v>2093.89095210065</v>
@@ -1528,7 +1528,7 @@
         <v>1217.715307419696</v>
       </c>
       <c r="H6" s="35" t="n">
-        <v>1125.139614400777</v>
+        <v>1110.545019820355</v>
       </c>
       <c r="I6" s="35" t="n">
         <v>852.1056303154498</v>
@@ -1569,7 +1569,7 @@
         <v>2105.91594721014</v>
       </c>
       <c r="H7" s="35" t="n">
-        <v>782.4450070208028</v>
+        <v>816.9741376043581</v>
       </c>
       <c r="I7" s="35" t="n">
         <v>1356.35062941391</v>
@@ -1610,7 +1610,7 @@
         <v>1937.226684229344</v>
       </c>
       <c r="H8" s="35" t="n">
-        <v>1432.784628468764</v>
+        <v>1455.288174287584</v>
       </c>
       <c r="I8" s="35" t="n">
         <v>1464.698970511554</v>
@@ -1651,7 +1651,7 @@
         <v>345.5367123230465</v>
       </c>
       <c r="H9" s="35" t="n">
-        <v>228.3356410895417</v>
+        <v>232.0502770563494</v>
       </c>
       <c r="I9" s="35" t="n">
         <v>259.0603361045289</v>
@@ -1692,7 +1692,7 @@
         <v>1075.844277632001</v>
       </c>
       <c r="H10" s="35" t="n">
-        <v>512.7869011515177</v>
+        <v>537.2797770286651</v>
       </c>
       <c r="I10" s="35" t="n">
         <v>1036.221280441298</v>
@@ -1733,7 +1733,7 @@
         <v>2119.52449650215</v>
       </c>
       <c r="H11" s="35" t="n">
-        <v>1707.732487744382</v>
+        <v>1708.093138162858</v>
       </c>
       <c r="I11" s="35" t="n">
         <v>2054.998366180861</v>
@@ -1774,7 +1774,7 @@
         <v>1078.784008134861</v>
       </c>
       <c r="H12" s="35" t="n">
-        <v>1580.532976974313</v>
+        <v>1570.296161854369</v>
       </c>
       <c r="I12" s="35" t="n">
         <v>1382.812148553971</v>
@@ -1815,7 +1815,7 @@
         <v>1090.583745727621</v>
       </c>
       <c r="H13" s="35" t="n">
-        <v>761.7126636085532</v>
+        <v>804.9809359057639</v>
       </c>
       <c r="I13" s="35" t="n">
         <v>983.9574871137551</v>
@@ -1856,7 +1856,7 @@
         <v>1216.088895856651</v>
       </c>
       <c r="H14" s="35" t="n">
-        <v>582.030392876443</v>
+        <v>570.7512848138058</v>
       </c>
       <c r="I14" s="35" t="n">
         <v>1940.060441839825</v>
@@ -1897,7 +1897,7 @@
         <v>246.6252247066325</v>
       </c>
       <c r="H15" s="35" t="n">
-        <v>163.8159310956179</v>
+        <v>168.6948157559068</v>
       </c>
       <c r="I15" s="35" t="n">
         <v>149.2759875232221</v>
@@ -1938,7 +1938,7 @@
         <v>1050.918637090984</v>
       </c>
       <c r="H16" s="35" t="n">
-        <v>1028.710489673385</v>
+        <v>1000.897800237597</v>
       </c>
       <c r="I16" s="35" t="n">
         <v>954.225539752419</v>
@@ -1979,7 +1979,7 @@
         <v>1623.297962092956</v>
       </c>
       <c r="H17" s="35" t="n">
-        <v>1923.746639273764</v>
+        <v>1924.84621065964</v>
       </c>
       <c r="I17" s="35" t="n">
         <v>1450.854826507385</v>
@@ -2020,7 +2020,7 @@
         <v>3516.719813419875</v>
       </c>
       <c r="H18" s="35" t="n">
-        <v>4409.234229542084</v>
+        <v>4400.800850653997</v>
       </c>
       <c r="I18" s="35" t="n">
         <v>3407.580909091359</v>
@@ -2061,7 +2061,7 @@
         <v>1733.627651320199</v>
       </c>
       <c r="H19" s="35" t="n">
-        <v>1807.925251362078</v>
+        <v>1820.495600641051</v>
       </c>
       <c r="I19" s="35" t="n">
         <v>2622.066542977747</v>
@@ -2102,7 +2102,7 @@
         <v>849.6769813029938</v>
       </c>
       <c r="H20" s="35" t="n">
-        <v>985.2552983823412</v>
+        <v>972.4931883765348</v>
       </c>
       <c r="I20" s="35" t="n">
         <v>703.101939620467</v>
@@ -2214,7 +2214,7 @@
         <v>68.69003876798844</v>
       </c>
       <c r="H25" s="36" t="n">
-        <v>23.10911292273983</v>
+        <v>29.64254553870305</v>
       </c>
       <c r="I25" s="36" t="n">
         <v>22.26514293693651</v>
@@ -2252,7 +2252,7 @@
         <v>-4.27354939043077</v>
       </c>
       <c r="H26" s="36" t="n">
-        <v>-72.76971423318405</v>
+        <v>-72.70563178000242</v>
       </c>
       <c r="I26" s="36" t="n">
         <v>2.647474148869351</v>
@@ -2290,7 +2290,7 @@
         <v>31.25100713804224</v>
       </c>
       <c r="H27" s="36" t="n">
-        <v>21.27276930921647</v>
+        <v>19.6996961731722</v>
       </c>
       <c r="I27" s="36" t="n">
         <v>-8.156100621019334</v>
@@ -2328,7 +2328,7 @@
         <v>52.6179140483064</v>
       </c>
       <c r="H28" s="36" t="n">
-        <v>-43.29539838129567</v>
+        <v>-40.79303645628863</v>
       </c>
       <c r="I28" s="36" t="n">
         <v>-1.703862372336926</v>
@@ -2366,7 +2366,7 @@
         <v>41.22806766178572</v>
       </c>
       <c r="H29" s="36" t="n">
-        <v>4.453137106487136</v>
+        <v>6.093694877760371</v>
       </c>
       <c r="I29" s="36" t="n">
         <v>6.779762531427293</v>
@@ -2404,7 +2404,7 @@
         <v>74.02255312421833</v>
       </c>
       <c r="H30" s="36" t="n">
-        <v>14.99661197941816</v>
+        <v>16.86741300233976</v>
       </c>
       <c r="I30" s="36" t="n">
         <v>30.47048112207599</v>
@@ -2442,7 +2442,7 @@
         <v>-18.28344971079963</v>
       </c>
       <c r="H31" s="36" t="n">
-        <v>-61.05089048033732</v>
+        <v>-59.19051592153274</v>
       </c>
       <c r="I31" s="36" t="n">
         <v>-21.29304385919226</v>
@@ -2480,7 +2480,7 @@
         <v>0.5227490108479224</v>
       </c>
       <c r="H32" s="36" t="n">
-        <v>-19.00732238457276</v>
+        <v>-18.99021780684458</v>
       </c>
       <c r="I32" s="36" t="n">
         <v>-2.537533620295328</v>
@@ -2518,7 +2518,7 @@
         <v>-6.562652756210437</v>
       </c>
       <c r="H33" s="36" t="n">
-        <v>36.89562274392504</v>
+        <v>36.0089755172143</v>
       </c>
       <c r="I33" s="36" t="n">
         <v>19.77031354103625</v>
@@ -2556,7 +2556,7 @@
         <v>28.70951507435355</v>
       </c>
       <c r="H34" s="36" t="n">
-        <v>-10.10349462558653</v>
+        <v>-4.997019889193404</v>
       </c>
       <c r="I34" s="36" t="n">
         <v>16.12559926399367</v>
@@ -2594,7 +2594,7 @@
         <v>-33.24624369916566</v>
       </c>
       <c r="H35" s="36" t="n">
-        <v>-68.05108973683714</v>
+        <v>-68.67022443453018</v>
       </c>
       <c r="I35" s="36" t="n">
         <v>6.494124224558738</v>
@@ -2632,7 +2632,7 @@
         <v>17.04974516602368</v>
       </c>
       <c r="H36" s="36" t="n">
-        <v>-22.25202019912726</v>
+        <v>-19.93647357626845</v>
       </c>
       <c r="I36" s="36" t="n">
         <v>-29.15276075355244</v>
@@ -2670,7 +2670,7 @@
         <v>-12.16656389197989</v>
       </c>
       <c r="H37" s="36" t="n">
-        <v>-14.0226713283088</v>
+        <v>-16.34719388822131</v>
       </c>
       <c r="I37" s="36" t="n">
         <v>-20.24795733903337</v>
@@ -2708,7 +2708,7 @@
         <v>-6.234333377151083</v>
       </c>
       <c r="H38" s="36" t="n">
-        <v>11.1203181776929</v>
+        <v>11.18383211438456</v>
       </c>
       <c r="I38" s="36" t="n">
         <v>-16.19507129483321</v>
@@ -2746,7 +2746,7 @@
         <v>-8.151625850031591</v>
       </c>
       <c r="H39" s="36" t="n">
-        <v>15.1587322039172</v>
+        <v>14.93847236504531</v>
       </c>
       <c r="I39" s="36" t="n">
         <v>-11.00207497618331</v>
@@ -2784,7 +2784,7 @@
         <v>-0.1408218127160009</v>
       </c>
       <c r="H40" s="36" t="n">
-        <v>4.138815326100731</v>
+        <v>4.8628835812243</v>
       </c>
       <c r="I40" s="36" t="n">
         <v>51.03439884264372</v>
@@ -2822,7 +2822,7 @@
         <v>-50.29851021472956</v>
       </c>
       <c r="H41" s="36" t="n">
-        <v>-42.36791483589533</v>
+        <v>-43.11442897485597</v>
       </c>
       <c r="I41" s="36" t="n">
         <v>-58.87235427225367</v>
@@ -3044,16 +3044,16 @@
         <v>223795.0176119162</v>
       </c>
       <c r="R4" s="40" t="n">
-        <v>7034.368899741121</v>
+        <v>7032.6650709678</v>
       </c>
       <c r="S4" s="40" t="n">
         <v>338765.0803665607</v>
       </c>
       <c r="T4" s="40" t="n">
-        <v>347038.6938929957</v>
+        <v>347036.9900642224</v>
       </c>
       <c r="U4" s="37" t="n">
-        <v>-15.15460825529512</v>
+        <v>-15.15502481408893</v>
       </c>
     </row>
     <row r="5">
@@ -3109,16 +3109,16 @@
         <v>1731146.785989288</v>
       </c>
       <c r="R5" s="40" t="n">
-        <v>307860.8460359017</v>
+        <v>307442.6849611326</v>
       </c>
       <c r="S5" s="40" t="n">
         <v>638495.8317639165</v>
       </c>
       <c r="T5" s="40" t="n">
-        <v>938737.7389709837</v>
+        <v>938319.5778962146</v>
       </c>
       <c r="U5" s="37" t="n">
-        <v>-64.30505690462401</v>
+        <v>-64.32095723029425</v>
       </c>
     </row>
     <row r="6">
@@ -3174,16 +3174,16 @@
         <v>584926.7958949648</v>
       </c>
       <c r="R6" s="40" t="n">
-        <v>516426.2290141381</v>
+        <v>515587.6526728149</v>
       </c>
       <c r="S6" s="40" t="n">
         <v>573614.3093442855</v>
       </c>
       <c r="T6" s="40" t="n">
-        <v>1092115.468371972</v>
+        <v>1091276.892030649</v>
       </c>
       <c r="U6" s="37" t="n">
-        <v>2.044969450664781</v>
+        <v>1.966614643311005</v>
       </c>
     </row>
     <row r="7">
@@ -3239,16 +3239,16 @@
         <v>987444.370965802</v>
       </c>
       <c r="R7" s="40" t="n">
-        <v>58449.00722249777</v>
+        <v>58423.52228916512</v>
       </c>
       <c r="S7" s="40" t="n">
         <v>717174.0210356977</v>
       </c>
       <c r="T7" s="40" t="n">
-        <v>775662.7048455855</v>
+        <v>775637.2199122529</v>
       </c>
       <c r="U7" s="37" t="n">
-        <v>-54.46792802818477</v>
+        <v>-54.46942401582405</v>
       </c>
     </row>
     <row r="8">
@@ -3304,16 +3304,16 @@
         <v>831996.1678874366</v>
       </c>
       <c r="R8" s="40" t="n">
-        <v>486827.7445076825</v>
+        <v>485934.2990438922</v>
       </c>
       <c r="S8" s="40" t="n">
         <v>1117528.146282031</v>
       </c>
       <c r="T8" s="40" t="n">
-        <v>1614844.56656084</v>
+        <v>1613951.121097049</v>
       </c>
       <c r="U8" s="37" t="n">
-        <v>-12.21934303520699</v>
+        <v>-12.26790946159734</v>
       </c>
     </row>
     <row r="9">
@@ -3369,16 +3369,16 @@
         <v>183076.3816710717</v>
       </c>
       <c r="R9" s="40" t="n">
-        <v>56560.4981316346</v>
+        <v>56427.79038137274</v>
       </c>
       <c r="S9" s="40" t="n">
         <v>219235.7465619491</v>
       </c>
       <c r="T9" s="40" t="n">
-        <v>276055.1116522022</v>
+        <v>275922.4039019403</v>
       </c>
       <c r="U9" s="37" t="n">
-        <v>-15.15791257225437</v>
+        <v>-15.19869864023432</v>
       </c>
     </row>
     <row r="10">
@@ -3434,16 +3434,16 @@
         <v>650385.3131989896</v>
       </c>
       <c r="R10" s="40" t="n">
-        <v>38679.04925274325</v>
+        <v>38601.6389769039</v>
       </c>
       <c r="S10" s="40" t="n">
         <v>749431.578620812</v>
       </c>
       <c r="T10" s="40" t="n">
-        <v>792121.3311342841</v>
+        <v>792043.9208584448</v>
       </c>
       <c r="U10" s="37" t="n">
-        <v>-39.13667446901931</v>
+        <v>-39.142622354315</v>
       </c>
     </row>
     <row r="11">
@@ -3499,16 +3499,16 @@
         <v>1250306.901376196</v>
       </c>
       <c r="R11" s="40" t="n">
-        <v>1130026.138226878</v>
+        <v>1128248.733642917</v>
       </c>
       <c r="S11" s="40" t="n">
         <v>1191270.093712525</v>
       </c>
       <c r="T11" s="40" t="n">
-        <v>2305970.369208368</v>
+        <v>2304192.964624406</v>
       </c>
       <c r="U11" s="37" t="n">
-        <v>-10.65737300753434</v>
+        <v>-10.72623685629839</v>
       </c>
     </row>
     <row r="12">
@@ -3564,16 +3564,16 @@
         <v>800962.2753742293</v>
       </c>
       <c r="R12" s="40" t="n">
-        <v>1560882.567371651</v>
+        <v>1558547.392683348</v>
       </c>
       <c r="S12" s="40" t="n">
         <v>1052956.818313675</v>
       </c>
       <c r="T12" s="40" t="n">
-        <v>2623659.574156143</v>
+        <v>2621324.39946784</v>
       </c>
       <c r="U12" s="37" t="n">
-        <v>51.06392826366002</v>
+        <v>50.92947459250861</v>
       </c>
     </row>
     <row r="13">
@@ -3629,16 +3629,16 @@
         <v>552101.8239241685</v>
       </c>
       <c r="R13" s="40" t="n">
-        <v>11704.87524284939</v>
+        <v>11679.63197050408</v>
       </c>
       <c r="S13" s="40" t="n">
         <v>1040262.573737449</v>
       </c>
       <c r="T13" s="40" t="n">
-        <v>1081083.786740756</v>
+        <v>1081058.543468411</v>
       </c>
       <c r="U13" s="37" t="n">
-        <v>-12.5218689107271</v>
+        <v>-12.52391152233077</v>
       </c>
     </row>
     <row r="14">
@@ -3694,16 +3694,16 @@
         <v>1478954.538372993</v>
       </c>
       <c r="R14" s="40" t="n">
-        <v>752246.0730030508</v>
+        <v>751106.1036434649</v>
       </c>
       <c r="S14" s="40" t="n">
         <v>596912.9762623194</v>
       </c>
       <c r="T14" s="40" t="n">
-        <v>1339960.945338871</v>
+        <v>1338820.975979285</v>
       </c>
       <c r="U14" s="37" t="n">
-        <v>-45.00877975444676</v>
+        <v>-45.05556343597437</v>
       </c>
     </row>
     <row r="15">
@@ -3759,16 +3759,16 @@
         <v>100907.4186907174</v>
       </c>
       <c r="R15" s="40" t="n">
-        <v>16072.55736896905</v>
+        <v>16033.99914779184</v>
       </c>
       <c r="S15" s="40" t="n">
         <v>146545.5591579213</v>
       </c>
       <c r="T15" s="40" t="n">
-        <v>162708.0982788303</v>
+        <v>162669.5400576531</v>
       </c>
       <c r="U15" s="37" t="n">
-        <v>-13.21679345940526</v>
+        <v>-13.23735916023795</v>
       </c>
     </row>
     <row r="16">
@@ -3824,16 +3824,16 @@
         <v>734886.085373234</v>
       </c>
       <c r="R16" s="40" t="n">
-        <v>848369.7524061274</v>
+        <v>846982.2317353879</v>
       </c>
       <c r="S16" s="40" t="n">
         <v>396973.1924639251</v>
       </c>
       <c r="T16" s="40" t="n">
-        <v>1244602.212880934</v>
+        <v>1243214.692210195</v>
       </c>
       <c r="U16" s="37" t="n">
-        <v>3.847491217362627</v>
+        <v>3.731718853166846</v>
       </c>
     </row>
     <row r="17">
@@ -3889,16 +3889,16 @@
         <v>931291.1409283208</v>
       </c>
       <c r="R17" s="40" t="n">
-        <v>1171527.49450492</v>
+        <v>1169639.541726666</v>
       </c>
       <c r="S17" s="40" t="n">
         <v>1149519.910123474</v>
       </c>
       <c r="T17" s="40" t="n">
-        <v>2347305.649533936</v>
+        <v>2345417.696755682</v>
       </c>
       <c r="U17" s="37" t="n">
-        <v>28.81373169480421</v>
+        <v>28.71012599578554</v>
       </c>
     </row>
     <row r="18">
@@ -3954,16 +3954,16 @@
         <v>2177088.604877107</v>
       </c>
       <c r="R18" s="40" t="n">
-        <v>4221634.661930383</v>
+        <v>4216057.928948273</v>
       </c>
       <c r="S18" s="40" t="n">
         <v>1270426.243885216</v>
       </c>
       <c r="T18" s="40" t="n">
-        <v>5386440.818376753</v>
+        <v>5380864.085394643</v>
       </c>
       <c r="U18" s="37" t="n">
-        <v>25.85549806132748</v>
+        <v>25.72519634063949</v>
       </c>
     </row>
     <row r="19">
@@ -4019,16 +4019,16 @@
         <v>1594652.173291156</v>
       </c>
       <c r="R19" s="40" t="n">
-        <v>1796724.208701453</v>
+        <v>1794108.92670873</v>
       </c>
       <c r="S19" s="40" t="n">
         <v>1914967.298411852</v>
       </c>
       <c r="T19" s="40" t="n">
-        <v>3786075.430069988</v>
+        <v>3783460.148077264</v>
       </c>
       <c r="U19" s="37" t="n">
-        <v>14.96404333025639</v>
+        <v>14.88463038725362</v>
       </c>
     </row>
     <row r="20">
@@ -4084,16 +4084,16 @@
         <v>449214.0917825571</v>
       </c>
       <c r="R20" s="40" t="n">
-        <v>493753.524919103</v>
+        <v>493052.450341224</v>
       </c>
       <c r="S20" s="40" t="n">
         <v>600716.3697009798</v>
       </c>
       <c r="T20" s="40" t="n">
-        <v>1098779.041767157</v>
+        <v>1098077.967189278</v>
       </c>
       <c r="U20" s="37" t="n">
-        <v>24.42525733318537</v>
+        <v>24.34586795511529</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove a vazao de base do modelo: MUSLE so com escoamento direto (lambda 0,20)
Decisao com o orientador (26/10/2026): a vazao de base nao produz erosao nas
encostas, entao o termo empirico de base saiu. Modelo adotado:
Scripts/calcular_sy_so_direto.py (SY = c * soma E_unit; calculado com Q do
SCS-CN e forcado com Q reescalado ao escoamento direto medido).

- Tabelas, figuras, mapas, escada do gargalo, Apendice B e planilha
  comparativa refeitos; fig_decomposicao.png removida, fig_volume_direto.png nova
- Notas secao 27 e README com o ponto de retomada
- Lista de mudancas para o Google Doc em
  Notas Claude/mudancas_docs_sem_base_26-10.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Comparacao_Modelos_TCC.xlsx
+++ b/Comparacao_Modelos_TCC.xlsx
@@ -598,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -966,163 +966,163 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>ADOTADO — Espacializada — Q = escoamento direto (λ = 0,20) + vazão de base prevista</t>
+          <t>ADOTADO — Espacializada — calculado: Q = só escoamento direto do SCS-CN (λ = 0,20)</t>
         </is>
       </c>
       <c r="B10" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>0.01465768957838539</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>-0.1430610598761948</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>-1.111271232572765</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>0.8076337504346727</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <v>-43.53950662539768</v>
+      </c>
+      <c r="J10" s="17" t="n">
+        <v>-56.01578682027758</v>
+      </c>
+      <c r="K10" s="17" t="n">
+        <v>60.61013891893332</v>
+      </c>
+      <c r="L10" s="16" t="n">
+        <v>-0.7833807874705723</v>
+      </c>
+      <c r="M10" s="16" t="n">
+        <v>-7.681737055638786</v>
+      </c>
+      <c r="N10" s="13" t="inlineStr">
+        <is>
+          <t>SY = c·ΣE_unit, com Q de cada pixel pelo SCS-CN (CN-I, λ = 0,20), sem termo de vazão de base (decisão de 26/10/2026). Aqui c por mínimos quadrados lineares, como nas demais linhas; no texto do TCC c é calibrado em log (tab_resultados.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>ADOTADO — Espacializada — forçado: Q reescalado para o escoamento direto medido</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Sim (volume direto)</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>0.02393903917940962</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>0.8004067054076534</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>0.7878135588475967</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>0.953407941825132</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <v>-7.441827102344136</v>
+      </c>
+      <c r="J11" s="17" t="n">
+        <v>-10.93578435733297</v>
+      </c>
+      <c r="K11" s="17" t="n">
+        <v>28.33924567441559</v>
+      </c>
+      <c r="L11" s="16" t="n">
+        <v>0.5885851313896476</v>
+      </c>
+      <c r="M11" s="16" t="n">
+        <v>0.4765633117073207</v>
+      </c>
+      <c r="N11" s="13" t="inlineStr">
+        <is>
+          <t>Q de cada pixel reescalado para o escoamento direto medido do evento (T_R − ΣBt·3600; limite Q ≤ chuva). Sem termo de base. Não é previsão: usa o volume medido. c por mínimos quadrados lineares nesta planilha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Não adotado (até 26/10/2026) — Espacializada — Q = escoamento direto (λ = 0,20) + vazão de base prevista</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Parcial (Qb inicial e duração)</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E12" s="15" t="n">
         <v>0.01021554737345453</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F12" s="16" t="n">
         <v>0.5014561479980195</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G12" s="16" t="n">
         <v>0.3804165146048779</v>
       </c>
-      <c r="H10" s="16" t="n">
+      <c r="H12" s="16" t="n">
         <v>0.8926167512266159</v>
       </c>
-      <c r="I10" s="17" t="n">
+      <c r="I12" s="17" t="n">
         <v>-16.14184757409659</v>
       </c>
-      <c r="J10" s="17" t="n">
+      <c r="J12" s="17" t="n">
         <v>-12.08513115046434</v>
       </c>
-      <c r="K10" s="17" t="n">
+      <c r="K12" s="17" t="n">
         <v>28.47307387632832</v>
       </c>
-      <c r="L10" s="16" t="n">
+      <c r="L12" s="16" t="n">
         <v>0.07702056088139086</v>
       </c>
-      <c r="M10" s="16" t="n">
+      <c r="M12" s="16" t="n">
         <v>0.567804501948117</v>
       </c>
-      <c r="N10" s="13" t="inlineStr">
+      <c r="N12" s="13" t="inlineStr">
         <is>
           <t>Q do pixel = SCS-CN (CN-I, λ = 0,20) + lâmina de base uniforme = kb·Qb_inicio·duração (kb = 1,93). LOO aninhado (kb e c refeitos sem o evento). A duração é a da janela observada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Sem MUSLE — SY = c · volume total medido (T_R)</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>Sim (volume)</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E11" s="20" t="n">
-        <v>0.0007961895562554518</v>
-      </c>
-      <c r="F11" s="21" t="n">
-        <v>0.8090940590219937</v>
-      </c>
-      <c r="G11" s="21" t="n">
-        <v>0.7653444578703972</v>
-      </c>
-      <c r="H11" s="21" t="n">
-        <v>0.9507257698920797</v>
-      </c>
-      <c r="I11" s="22" t="n">
-        <v>-3.391753649336037</v>
-      </c>
-      <c r="J11" s="22" t="n">
-        <v>-0.7984389704210787</v>
-      </c>
-      <c r="K11" s="22" t="n">
-        <v>19.10282680707302</v>
-      </c>
-      <c r="L11" s="21" t="n">
-        <v>0.6460347620386332</v>
-      </c>
-      <c r="M11" s="21" t="n">
-        <v>0.872949845816107</v>
-      </c>
-      <c r="N11" s="18" t="inlineStr">
-        <is>
-          <t>Referência trivial: sedimento proporcional ao volume total medido. Empata ou supera os modelos espacializados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Sem MUSLE — SY = c · escoamento direto medido</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>Sim (volume)</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="n">
-        <v>0.001498452605952412</v>
-      </c>
-      <c r="F12" s="21" t="n">
-        <v>0.7829694944221395</v>
-      </c>
-      <c r="G12" s="21" t="n">
-        <v>0.7326575009900256</v>
-      </c>
-      <c r="H12" s="21" t="n">
-        <v>0.944017090866361</v>
-      </c>
-      <c r="I12" s="22" t="n">
-        <v>-4.087214215008808</v>
-      </c>
-      <c r="J12" s="22" t="n">
-        <v>-1.378850569568219</v>
-      </c>
-      <c r="K12" s="22" t="n">
-        <v>20.40253847958454</v>
-      </c>
-      <c r="L12" s="21" t="n">
-        <v>0.623484423390292</v>
-      </c>
-      <c r="M12" s="21" t="n">
-        <v>0.8619387224365678</v>
-      </c>
-      <c r="N12" s="18" t="inlineStr">
-        <is>
-          <t>Mesma referência, com o escoamento direto (T_R − Σ Bt·3600).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>Sem MUSLE — SY = c · chuva do evento</t>
+          <t>Sem MUSLE — SY = c · volume total medido (T_R)</t>
         </is>
       </c>
       <c r="B13" s="19" t="n">
@@ -1130,188 +1130,292 @@
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
+          <t>Sim (volume)</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>0.0007961895562554518</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>0.8090940590219937</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>0.7653444578703972</v>
+      </c>
+      <c r="H13" s="21" t="n">
+        <v>0.9507257698920797</v>
+      </c>
+      <c r="I13" s="22" t="n">
+        <v>-3.391753649336037</v>
+      </c>
+      <c r="J13" s="22" t="n">
+        <v>-0.7984389704210787</v>
+      </c>
+      <c r="K13" s="22" t="n">
+        <v>19.10282680707302</v>
+      </c>
+      <c r="L13" s="21" t="n">
+        <v>0.6460347620386332</v>
+      </c>
+      <c r="M13" s="21" t="n">
+        <v>0.872949845816107</v>
+      </c>
+      <c r="N13" s="18" t="inlineStr">
+        <is>
+          <t>Referência trivial: sedimento proporcional ao volume total medido. Empata ou supera os modelos espacializados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Sem MUSLE — SY = c · escoamento direto medido</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Sim (volume)</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="n">
+        <v>0.001498452605952412</v>
+      </c>
+      <c r="F14" s="21" t="n">
+        <v>0.7829694944221395</v>
+      </c>
+      <c r="G14" s="21" t="n">
+        <v>0.7326575009900256</v>
+      </c>
+      <c r="H14" s="21" t="n">
+        <v>0.944017090866361</v>
+      </c>
+      <c r="I14" s="22" t="n">
+        <v>-4.087214215008808</v>
+      </c>
+      <c r="J14" s="22" t="n">
+        <v>-1.378850569568219</v>
+      </c>
+      <c r="K14" s="22" t="n">
+        <v>20.40253847958454</v>
+      </c>
+      <c r="L14" s="21" t="n">
+        <v>0.623484423390292</v>
+      </c>
+      <c r="M14" s="21" t="n">
+        <v>0.8619387224365678</v>
+      </c>
+      <c r="N14" s="18" t="inlineStr">
+        <is>
+          <t>Mesma referência, com o escoamento direto (T_R − Σ Bt·3600).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Sem MUSLE — SY = c · chuva do evento</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
           <t>Sim (chuva)</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="E13" s="20" t="n">
+      <c r="E15" s="20" t="n">
         <v>22.32215182996425</v>
       </c>
-      <c r="F13" s="21" t="n">
+      <c r="F15" s="21" t="n">
         <v>0.670573753905237</v>
       </c>
-      <c r="G13" s="21" t="n">
+      <c r="G15" s="21" t="n">
         <v>0.6050248690021753</v>
       </c>
-      <c r="H13" s="21" t="n">
+      <c r="H15" s="21" t="n">
         <v>0.8930732205069412</v>
       </c>
-      <c r="I13" s="22" t="n">
+      <c r="I15" s="22" t="n">
         <v>0.3555526316416786</v>
       </c>
-      <c r="J13" s="22" t="n">
+      <c r="J15" s="22" t="n">
         <v>31.56009507155892</v>
       </c>
-      <c r="K13" s="22" t="n">
+      <c r="K15" s="22" t="n">
         <v>55.83818107257348</v>
       </c>
-      <c r="L13" s="21" t="n">
+      <c r="L15" s="21" t="n">
         <v>0.4322127199602186</v>
       </c>
-      <c r="M13" s="21" t="n">
+      <c r="M15" s="21" t="n">
         <v>0.5638685217717554</v>
       </c>
-      <c r="N13" s="18" t="inlineStr">
+      <c r="N15" s="18" t="inlineStr">
         <is>
           <t>Referência trivial: sedimento proporcional à lâmina de chuva do evento (não usa vazão).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="23" t="inlineStr">
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>Espacializada — α e β livres (experimento, não adotado)</t>
         </is>
       </c>
-      <c r="B14" s="24" t="n">
+      <c r="B16" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C16" s="24" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="D14" s="24" t="inlineStr">
+      <c r="D16" s="24" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="E14" s="24" t="n"/>
-      <c r="F14" s="25" t="n">
+      <c r="E16" s="24" t="n"/>
+      <c r="F16" s="25" t="n">
         <v>0.6120927741732798</v>
       </c>
-      <c r="G14" s="24" t="inlineStr">
+      <c r="G16" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H14" s="25" t="n">
+      <c r="H16" s="25" t="n">
         <v>0.8779670710651121</v>
       </c>
-      <c r="I14" s="26" t="n">
+      <c r="I16" s="26" t="n">
         <v>-1.359787660971752</v>
       </c>
-      <c r="J14" s="26" t="n">
+      <c r="J16" s="26" t="n">
         <v>29.23856688755154</v>
       </c>
-      <c r="K14" s="26" t="n">
+      <c r="K16" s="26" t="n">
         <v>57.85399063634824</v>
       </c>
-      <c r="L14" s="25" t="n">
+      <c r="L16" s="25" t="n">
         <v>0.2794748944469283</v>
       </c>
-      <c r="M14" s="25" t="n">
+      <c r="M16" s="25" t="n">
         <v>0.5037305280139199</v>
       </c>
-      <c r="N14" s="23" t="inlineStr">
+      <c r="N16" s="23" t="inlineStr">
         <is>
           <t>α = 4,22 e β = 0,28 ajustados na fórmula por pixel (NSE bruto). Só in-sample; instável em eventos pequenos.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="23" t="inlineStr">
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>Espacializada — com FCI/DSC de Hao (descartado)</t>
         </is>
       </c>
-      <c r="B15" s="24" t="n">
+      <c r="B17" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="24" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="D15" s="24" t="inlineStr">
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="E15" s="24" t="n"/>
-      <c r="F15" s="25" t="n">
+      <c r="E17" s="24" t="n"/>
+      <c r="F17" s="25" t="n">
         <v>0.2059722483388605</v>
       </c>
-      <c r="G15" s="24" t="inlineStr">
+      <c r="G17" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H15" s="25" t="n">
+      <c r="H17" s="25" t="n">
         <v>0.8492652457985379</v>
       </c>
-      <c r="I15" s="26" t="n">
+      <c r="I17" s="26" t="n">
         <v>-27.60542986665604</v>
       </c>
-      <c r="J15" s="26" t="n">
+      <c r="J17" s="26" t="n">
         <v>-30.81712256272602</v>
       </c>
-      <c r="K15" s="26" t="n">
+      <c r="K17" s="26" t="n">
         <v>46.47290066656894</v>
       </c>
-      <c r="L15" s="25" t="n">
+      <c r="L17" s="25" t="n">
         <v>-0.5201467513534836</v>
       </c>
-      <c r="M15" s="25" t="n">
+      <c r="M17" s="25" t="n">
         <v>-1.100415318018777</v>
       </c>
-      <c r="N15" s="23" t="inlineStr">
+      <c r="N17" s="23" t="inlineStr">
         <is>
           <t>Eq. 8 exata, objetivo NSE bruto: FCI₀ = 3,17 (limite da busca) e k = 4,90. Só in-sample; valores por evento arredondados.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="27" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>Legenda de cores</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>Referência</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="29" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>Concentrada (um D e um qp por evento)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="30" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
         <is>
           <t>Espacializada (pixel a pixel)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="31" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Referência sem MUSLE (modelo trivial)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="32" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>Experimento não adotado</t>
         </is>
@@ -1331,7 +1435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1347,6 +1451,8 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1394,30 +1500,40 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>ADOTADO — Espacializada — Q = escoamento direto (λ = 0,20) + vazão de base prevista</t>
+          <t>ADOTADO — Espacializada — calculado: Q = só escoamento direto do SCS-CN (λ = 0,20)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
+          <t>ADOTADO — Espacializada — forçado: Q reescalado para o escoamento direto medido</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Não adotado (até 26/10/2026) — Espacializada — Q = escoamento direto (λ = 0,20) + vazão de base prevista</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
           <t>Sem MUSLE — SY = c · volume total medido (T_R)</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · escoamento direto medido</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · chuva do evento</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Espacializada — α e β livres (experimento, não adotado)</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Espacializada — com FCI/DSC de Hao (descartado)</t>
         </is>
@@ -1446,21 +1562,27 @@
         <v>449.3170466927465</v>
       </c>
       <c r="H4" s="35" t="n">
+        <v>3.395812369796301</v>
+      </c>
+      <c r="I4" s="35" t="n">
+        <v>112.1412828113571</v>
+      </c>
+      <c r="J4" s="35" t="n">
         <v>345.3114725244459</v>
       </c>
-      <c r="I4" s="35" t="n">
+      <c r="K4" s="35" t="n">
         <v>325.6612740094749</v>
       </c>
-      <c r="J4" s="35" t="n">
+      <c r="L4" s="35" t="n">
         <v>335.3462273397419</v>
       </c>
-      <c r="K4" s="35" t="n">
+      <c r="M4" s="35" t="n">
         <v>521.5406672974292</v>
       </c>
-      <c r="L4" s="35" t="n">
+      <c r="N4" s="35" t="n">
         <v>402.31</v>
       </c>
-      <c r="M4" s="35" t="n">
+      <c r="O4" s="35" t="n">
         <v>44</v>
       </c>
     </row>
@@ -1487,21 +1609,27 @@
         <v>1952.709995741231</v>
       </c>
       <c r="H5" s="35" t="n">
+        <v>221.9471536947734</v>
+      </c>
+      <c r="I5" s="35" t="n">
+        <v>2446.152720547311</v>
+      </c>
+      <c r="J5" s="35" t="n">
         <v>556.7738625138491</v>
       </c>
-      <c r="I5" s="35" t="n">
+      <c r="K5" s="35" t="n">
         <v>2093.89095210065</v>
       </c>
-      <c r="J5" s="35" t="n">
+      <c r="L5" s="35" t="n">
         <v>2594.041412751792</v>
       </c>
-      <c r="K5" s="35" t="n">
+      <c r="M5" s="35" t="n">
         <v>1279.94063140894</v>
       </c>
-      <c r="L5" s="35" t="n">
+      <c r="N5" s="35" t="n">
         <v>1166.06</v>
       </c>
-      <c r="M5" s="35" t="n">
+      <c r="O5" s="35" t="n">
         <v>458</v>
       </c>
     </row>
@@ -1528,21 +1656,27 @@
         <v>1217.715307419696</v>
       </c>
       <c r="H6" s="35" t="n">
+        <v>715.2497859025611</v>
+      </c>
+      <c r="I6" s="35" t="n">
+        <v>1345.46939045668</v>
+      </c>
+      <c r="J6" s="35" t="n">
         <v>1110.545019820355</v>
       </c>
-      <c r="I6" s="35" t="n">
+      <c r="K6" s="35" t="n">
         <v>852.1056303154498</v>
       </c>
-      <c r="J6" s="35" t="n">
+      <c r="L6" s="35" t="n">
         <v>876.4850816002048</v>
       </c>
-      <c r="K6" s="35" t="n">
+      <c r="M6" s="35" t="n">
         <v>1460.56347873917</v>
       </c>
-      <c r="L6" s="35" t="n">
+      <c r="N6" s="35" t="n">
         <v>1774.47</v>
       </c>
-      <c r="M6" s="35" t="n">
+      <c r="O6" s="35" t="n">
         <v>1275</v>
       </c>
     </row>
@@ -1569,21 +1703,27 @@
         <v>2105.91594721014</v>
       </c>
       <c r="H7" s="35" t="n">
+        <v>45.54912984079175</v>
+      </c>
+      <c r="I7" s="35" t="n">
+        <v>1273.278586203443</v>
+      </c>
+      <c r="J7" s="35" t="n">
         <v>816.9741376043581</v>
       </c>
-      <c r="I7" s="35" t="n">
+      <c r="K7" s="35" t="n">
         <v>1356.35062941391</v>
       </c>
-      <c r="J7" s="35" t="n">
+      <c r="L7" s="35" t="n">
         <v>1479.638590906746</v>
       </c>
-      <c r="K7" s="35" t="n">
+      <c r="M7" s="35" t="n">
         <v>807.7466937250238</v>
       </c>
-      <c r="L7" s="35" t="n">
+      <c r="N7" s="35" t="n">
         <v>830.3200000000001</v>
       </c>
-      <c r="M7" s="35" t="n">
+      <c r="O7" s="35" t="n">
         <v>219</v>
       </c>
     </row>
@@ -1610,21 +1750,27 @@
         <v>1937.226684229344</v>
       </c>
       <c r="H8" s="35" t="n">
+        <v>583.6999398535477</v>
+      </c>
+      <c r="I8" s="35" t="n">
+        <v>1733.516766331042</v>
+      </c>
+      <c r="J8" s="35" t="n">
         <v>1455.288174287584</v>
       </c>
-      <c r="I8" s="35" t="n">
+      <c r="K8" s="35" t="n">
         <v>1464.698970511554</v>
       </c>
-      <c r="J8" s="35" t="n">
+      <c r="L8" s="35" t="n">
         <v>1246.70682591335</v>
       </c>
-      <c r="K8" s="35" t="n">
+      <c r="M8" s="35" t="n">
         <v>1359.650667409476</v>
       </c>
-      <c r="L8" s="35" t="n">
+      <c r="N8" s="35" t="n">
         <v>1512.46</v>
       </c>
-      <c r="M8" s="35" t="n">
+      <c r="O8" s="35" t="n">
         <v>993</v>
       </c>
     </row>
@@ -1651,21 +1797,27 @@
         <v>345.5367123230465</v>
       </c>
       <c r="H9" s="35" t="n">
+        <v>49.51079330413807</v>
+      </c>
+      <c r="I9" s="35" t="n">
+        <v>285.5869566669709</v>
+      </c>
+      <c r="J9" s="35" t="n">
         <v>232.0502770563494</v>
       </c>
-      <c r="I9" s="35" t="n">
+      <c r="K9" s="35" t="n">
         <v>259.0603361045289</v>
       </c>
-      <c r="J9" s="35" t="n">
+      <c r="L9" s="35" t="n">
         <v>274.3312812033558</v>
       </c>
-      <c r="K9" s="35" t="n">
+      <c r="M9" s="35" t="n">
         <v>769.0109774995045</v>
       </c>
-      <c r="L9" s="35" t="n">
+      <c r="N9" s="35" t="n">
         <v>798.67</v>
       </c>
-      <c r="M9" s="35" t="n">
+      <c r="O9" s="35" t="n">
         <v>255</v>
       </c>
     </row>
@@ -1692,21 +1844,27 @@
         <v>1075.844277632001</v>
       </c>
       <c r="H10" s="35" t="n">
+        <v>19.57271851367251</v>
+      </c>
+      <c r="I10" s="35" t="n">
+        <v>588.6928725381608</v>
+      </c>
+      <c r="J10" s="35" t="n">
         <v>537.2797770286651</v>
       </c>
-      <c r="I10" s="35" t="n">
+      <c r="K10" s="35" t="n">
         <v>1036.221280441298</v>
       </c>
-      <c r="J10" s="35" t="n">
+      <c r="L10" s="35" t="n">
         <v>974.5715674362018</v>
       </c>
-      <c r="K10" s="35" t="n">
+      <c r="M10" s="35" t="n">
         <v>792.9220828686108</v>
       </c>
-      <c r="L10" s="35" t="n">
+      <c r="N10" s="35" t="n">
         <v>665.33</v>
       </c>
-      <c r="M10" s="35" t="n">
+      <c r="O10" s="35" t="n">
         <v>141</v>
       </c>
     </row>
@@ -1733,21 +1891,27 @@
         <v>2119.52449650215</v>
       </c>
       <c r="H11" s="35" t="n">
+        <v>1147.500617819254</v>
+      </c>
+      <c r="I11" s="35" t="n">
+        <v>2102.61282989047</v>
+      </c>
+      <c r="J11" s="35" t="n">
         <v>1708.093138162858</v>
       </c>
-      <c r="I11" s="35" t="n">
+      <c r="K11" s="35" t="n">
         <v>2054.998366180861</v>
       </c>
-      <c r="J11" s="35" t="n">
+      <c r="L11" s="35" t="n">
         <v>1873.525634607447</v>
       </c>
-      <c r="K11" s="35" t="n">
+      <c r="M11" s="35" t="n">
         <v>1842.362352711668</v>
       </c>
-      <c r="L11" s="35" t="n">
+      <c r="N11" s="35" t="n">
         <v>1864.47</v>
       </c>
-      <c r="M11" s="35" t="n">
+      <c r="O11" s="35" t="n">
         <v>1469</v>
       </c>
     </row>
@@ -1774,21 +1938,27 @@
         <v>1078.784008134861</v>
       </c>
       <c r="H12" s="35" t="n">
+        <v>1313.525572216108</v>
+      </c>
+      <c r="I12" s="35" t="n">
+        <v>1017.838378661586</v>
+      </c>
+      <c r="J12" s="35" t="n">
         <v>1570.296161854369</v>
       </c>
-      <c r="I12" s="35" t="n">
+      <c r="K12" s="35" t="n">
         <v>1382.812148553971</v>
       </c>
-      <c r="J12" s="35" t="n">
+      <c r="L12" s="35" t="n">
         <v>1200.204008804088</v>
       </c>
-      <c r="K12" s="35" t="n">
+      <c r="M12" s="35" t="n">
         <v>2074.59959813259</v>
       </c>
-      <c r="L12" s="35" t="n">
+      <c r="N12" s="35" t="n">
         <v>1893.59</v>
       </c>
-      <c r="M12" s="35" t="n">
+      <c r="O12" s="35" t="n">
         <v>1497</v>
       </c>
     </row>
@@ -1815,21 +1985,27 @@
         <v>1090.583745727621</v>
       </c>
       <c r="H13" s="35" t="n">
+        <v>4.1637881072344</v>
+      </c>
+      <c r="I13" s="35" t="n">
+        <v>145.7212013974608</v>
+      </c>
+      <c r="J13" s="35" t="n">
         <v>804.9809359057639</v>
       </c>
-      <c r="I13" s="35" t="n">
+      <c r="K13" s="35" t="n">
         <v>983.9574871137551</v>
       </c>
-      <c r="J13" s="35" t="n">
+      <c r="L13" s="35" t="n">
         <v>827.2984168102502</v>
       </c>
-      <c r="K13" s="35" t="n">
+      <c r="M13" s="35" t="n">
         <v>575.4290314409496</v>
       </c>
-      <c r="L13" s="35" t="n">
+      <c r="N13" s="35" t="n">
         <v>423.83</v>
       </c>
-      <c r="M13" s="35" t="n">
+      <c r="O13" s="35" t="n">
         <v>58</v>
       </c>
     </row>
@@ -1856,21 +2032,27 @@
         <v>1216.088895856651</v>
       </c>
       <c r="H14" s="35" t="n">
+        <v>439.7781609316646</v>
+      </c>
+      <c r="I14" s="35" t="n">
+        <v>1527.206571449622</v>
+      </c>
+      <c r="J14" s="35" t="n">
         <v>570.7512848138058</v>
       </c>
-      <c r="I14" s="35" t="n">
+      <c r="K14" s="35" t="n">
         <v>1940.060441839825</v>
       </c>
-      <c r="J14" s="35" t="n">
+      <c r="L14" s="35" t="n">
         <v>2216.143282110158</v>
       </c>
-      <c r="K14" s="35" t="n">
+      <c r="M14" s="35" t="n">
         <v>1652.72381593072</v>
       </c>
-      <c r="L14" s="35" t="n">
+      <c r="N14" s="35" t="n">
         <v>1297.32</v>
       </c>
-      <c r="M14" s="35" t="n">
+      <c r="O14" s="35" t="n">
         <v>600</v>
       </c>
     </row>
@@ -1897,21 +2079,27 @@
         <v>246.6252247066325</v>
       </c>
       <c r="H15" s="35" t="n">
+        <v>11.3477495965152</v>
+      </c>
+      <c r="I15" s="35" t="n">
+        <v>109.5947018190772</v>
+      </c>
+      <c r="J15" s="35" t="n">
         <v>168.6948157559068</v>
       </c>
-      <c r="I15" s="35" t="n">
+      <c r="K15" s="35" t="n">
         <v>149.2759875232221</v>
       </c>
-      <c r="J15" s="35" t="n">
+      <c r="L15" s="35" t="n">
         <v>151.2049844970366</v>
       </c>
-      <c r="K15" s="35" t="n">
+      <c r="M15" s="35" t="n">
         <v>529.6622290370957</v>
       </c>
-      <c r="L15" s="35" t="n">
+      <c r="N15" s="35" t="n">
         <v>535.14</v>
       </c>
-      <c r="M15" s="35" t="n">
+      <c r="O15" s="35" t="n">
         <v>127</v>
       </c>
     </row>
@@ -1938,21 +2126,27 @@
         <v>1050.918637090984</v>
       </c>
       <c r="H16" s="35" t="n">
+        <v>968.6623252219821</v>
+      </c>
+      <c r="I16" s="35" t="n">
+        <v>1349.462486031505</v>
+      </c>
+      <c r="J16" s="35" t="n">
         <v>1000.897800237597</v>
       </c>
-      <c r="I16" s="35" t="n">
+      <c r="K16" s="35" t="n">
         <v>954.225539752419</v>
       </c>
-      <c r="J16" s="35" t="n">
+      <c r="L16" s="35" t="n">
         <v>1101.191969705689</v>
       </c>
-      <c r="K16" s="35" t="n">
+      <c r="M16" s="35" t="n">
         <v>1671.536750534142</v>
       </c>
-      <c r="L16" s="35" t="n">
+      <c r="N16" s="35" t="n">
         <v>1806.8</v>
       </c>
-      <c r="M16" s="35" t="n">
+      <c r="O16" s="35" t="n">
         <v>1379</v>
       </c>
     </row>
@@ -1979,21 +2173,27 @@
         <v>1623.297962092956</v>
       </c>
       <c r="H17" s="35" t="n">
+        <v>1352.394474684254</v>
+      </c>
+      <c r="I17" s="35" t="n">
+        <v>1711.20493728039</v>
+      </c>
+      <c r="J17" s="35" t="n">
         <v>1924.84621065964</v>
       </c>
-      <c r="I17" s="35" t="n">
+      <c r="K17" s="35" t="n">
         <v>1450.854826507385</v>
       </c>
-      <c r="J17" s="35" t="n">
+      <c r="L17" s="35" t="n">
         <v>1395.495637024438</v>
       </c>
-      <c r="K17" s="35" t="n">
+      <c r="M17" s="35" t="n">
         <v>1834.958040560652</v>
       </c>
-      <c r="L17" s="35" t="n">
+      <c r="N17" s="35" t="n">
         <v>1969.22</v>
       </c>
-      <c r="M17" s="35" t="n">
+      <c r="O17" s="35" t="n">
         <v>1729</v>
       </c>
     </row>
@@ -2020,21 +2220,27 @@
         <v>3516.719813419875</v>
       </c>
       <c r="H18" s="35" t="n">
+        <v>4796.869212743336</v>
+      </c>
+      <c r="I18" s="35" t="n">
+        <v>3737.015958976279</v>
+      </c>
+      <c r="J18" s="35" t="n">
         <v>4400.800850653997</v>
       </c>
-      <c r="I18" s="35" t="n">
+      <c r="K18" s="35" t="n">
         <v>3407.580909091359</v>
       </c>
-      <c r="J18" s="35" t="n">
+      <c r="L18" s="35" t="n">
         <v>3262.264093367402</v>
       </c>
-      <c r="K18" s="35" t="n">
+      <c r="M18" s="35" t="n">
         <v>3112.21931817309</v>
       </c>
-      <c r="L18" s="35" t="n">
+      <c r="N18" s="35" t="n">
         <v>3132.09</v>
       </c>
-      <c r="M18" s="35" t="n">
+      <c r="O18" s="35" t="n">
         <v>4683</v>
       </c>
     </row>
@@ -2061,21 +2267,27 @@
         <v>1733.627651320199</v>
       </c>
       <c r="H19" s="35" t="n">
+        <v>1208.906982399343</v>
+      </c>
+      <c r="I19" s="35" t="n">
+        <v>1730.251773390043</v>
+      </c>
+      <c r="J19" s="35" t="n">
         <v>1820.495600641051</v>
       </c>
-      <c r="I19" s="35" t="n">
+      <c r="K19" s="35" t="n">
         <v>2622.066542977747</v>
       </c>
-      <c r="J19" s="35" t="n">
+      <c r="L19" s="35" t="n">
         <v>2389.51070465581</v>
       </c>
-      <c r="K19" s="35" t="n">
+      <c r="M19" s="35" t="n">
         <v>2180.37885993762</v>
       </c>
-      <c r="L19" s="35" t="n">
+      <c r="N19" s="35" t="n">
         <v>1783.68</v>
       </c>
-      <c r="M19" s="35" t="n">
+      <c r="O19" s="35" t="n">
         <v>1287</v>
       </c>
     </row>
@@ -2102,21 +2314,27 @@
         <v>849.6769813029938</v>
       </c>
       <c r="H20" s="35" t="n">
+        <v>581.3318826023811</v>
+      </c>
+      <c r="I20" s="35" t="n">
+        <v>855.4070352425226</v>
+      </c>
+      <c r="J20" s="35" t="n">
         <v>972.4931883765348</v>
       </c>
-      <c r="I20" s="35" t="n">
+      <c r="K20" s="35" t="n">
         <v>703.101939620467</v>
       </c>
-      <c r="J20" s="35" t="n">
+      <c r="L20" s="35" t="n">
         <v>673.1260264621188</v>
       </c>
-      <c r="K20" s="35" t="n">
+      <c r="M20" s="35" t="n">
         <v>1465.24989405988</v>
       </c>
-      <c r="L20" s="35" t="n">
+      <c r="N20" s="35" t="n">
         <v>1665.7</v>
       </c>
-      <c r="M20" s="35" t="n">
+      <c r="O20" s="35" t="n">
         <v>1049</v>
       </c>
     </row>
@@ -2165,30 +2383,40 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>ADOTADO — Espacializada — Q = escoamento direto (λ = 0,20) + vazão de base prevista</t>
+          <t>ADOTADO — Espacializada — calculado: Q = só escoamento direto do SCS-CN (λ = 0,20)</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
+          <t>ADOTADO — Espacializada — forçado: Q reescalado para o escoamento direto medido</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Não adotado (até 26/10/2026) — Espacializada — Q = escoamento direto (λ = 0,20) + vazão de base prevista</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
           <t>Sem MUSLE — SY = c · volume total medido (T_R)</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr">
+      <c r="L24" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · escoamento direto medido</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · chuva do evento</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>Espacializada — α e β livres (experimento, não adotado)</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="O24" s="3" t="inlineStr">
         <is>
           <t>Espacializada — com FCI/DSC de Hao (descartado)</t>
         </is>
@@ -2214,21 +2442,27 @@
         <v>68.69003876798844</v>
       </c>
       <c r="H25" s="36" t="n">
+        <v>-98.72508794285413</v>
+      </c>
+      <c r="I25" s="36" t="n">
+        <v>-57.89806444206479</v>
+      </c>
+      <c r="J25" s="36" t="n">
         <v>29.64254553870305</v>
       </c>
-      <c r="I25" s="36" t="n">
+      <c r="K25" s="36" t="n">
         <v>22.26514293693651</v>
       </c>
-      <c r="J25" s="36" t="n">
+      <c r="L25" s="36" t="n">
         <v>25.90122833537476</v>
       </c>
-      <c r="K25" s="36" t="n">
+      <c r="M25" s="36" t="n">
         <v>95.8054252182597</v>
       </c>
-      <c r="L25" s="36" t="n">
+      <c r="N25" s="36" t="n">
         <v>51.04187565613901</v>
       </c>
-      <c r="M25" s="36" t="n">
+      <c r="O25" s="36" t="n">
         <v>-83.48079210342742</v>
       </c>
     </row>
@@ -2252,21 +2486,27 @@
         <v>-4.27354939043077</v>
       </c>
       <c r="H26" s="36" t="n">
+        <v>-89.11962693260433</v>
+      </c>
+      <c r="I26" s="36" t="n">
+        <v>19.91617705528769</v>
+      </c>
+      <c r="J26" s="36" t="n">
         <v>-72.70563178000242</v>
       </c>
-      <c r="I26" s="36" t="n">
+      <c r="K26" s="36" t="n">
         <v>2.647474148869351</v>
       </c>
-      <c r="J26" s="36" t="n">
+      <c r="L26" s="36" t="n">
         <v>27.16602962986431</v>
       </c>
-      <c r="K26" s="36" t="n">
+      <c r="M26" s="36" t="n">
         <v>-37.25429075337954</v>
       </c>
-      <c r="L26" s="36" t="n">
+      <c r="N26" s="36" t="n">
         <v>-42.83698795968764</v>
       </c>
-      <c r="M26" s="36" t="n">
+      <c r="O26" s="36" t="n">
         <v>-77.54775953684796</v>
       </c>
     </row>
@@ -2290,21 +2530,27 @@
         <v>31.25100713804224</v>
       </c>
       <c r="H27" s="36" t="n">
+        <v>-22.90705866718269</v>
+      </c>
+      <c r="I27" s="36" t="n">
+        <v>45.02093510267608</v>
+      </c>
+      <c r="J27" s="36" t="n">
         <v>19.6996961731722</v>
       </c>
-      <c r="I27" s="36" t="n">
+      <c r="K27" s="36" t="n">
         <v>-8.156100621019334</v>
       </c>
-      <c r="J27" s="36" t="n">
+      <c r="L27" s="36" t="n">
         <v>-5.528370218765239</v>
       </c>
-      <c r="K27" s="36" t="n">
+      <c r="M27" s="36" t="n">
         <v>57.42631007880354</v>
       </c>
-      <c r="L27" s="36" t="n">
+      <c r="N27" s="36" t="n">
         <v>91.26061175148753</v>
       </c>
-      <c r="M27" s="36" t="n">
+      <c r="O27" s="36" t="n">
         <v>37.4254171573183</v>
       </c>
     </row>
@@ -2328,21 +2574,27 @@
         <v>52.6179140483064</v>
       </c>
       <c r="H28" s="36" t="n">
+        <v>-96.69900729313228</v>
+      </c>
+      <c r="I28" s="36" t="n">
+        <v>-7.724179549434214</v>
+      </c>
+      <c r="J28" s="36" t="n">
         <v>-40.79303645628863</v>
       </c>
-      <c r="I28" s="36" t="n">
+      <c r="K28" s="36" t="n">
         <v>-1.703862372336926</v>
       </c>
-      <c r="J28" s="36" t="n">
+      <c r="L28" s="36" t="n">
         <v>7.230944135601576</v>
       </c>
-      <c r="K28" s="36" t="n">
+      <c r="M28" s="36" t="n">
         <v>-41.46175888973972</v>
       </c>
-      <c r="L28" s="36" t="n">
+      <c r="N28" s="36" t="n">
         <v>-39.82584795918982</v>
       </c>
-      <c r="M28" s="36" t="n">
+      <c r="O28" s="36" t="n">
         <v>-84.12884273901938</v>
       </c>
     </row>
@@ -2366,21 +2618,27 @@
         <v>41.22806766178572</v>
       </c>
       <c r="H29" s="36" t="n">
+        <v>-57.44699612548916</v>
+      </c>
+      <c r="I29" s="36" t="n">
+        <v>26.37716853752386</v>
+      </c>
+      <c r="J29" s="36" t="n">
         <v>6.093694877760371</v>
       </c>
-      <c r="I29" s="36" t="n">
+      <c r="K29" s="36" t="n">
         <v>6.779762531427293</v>
       </c>
-      <c r="J29" s="36" t="n">
+      <c r="L29" s="36" t="n">
         <v>-9.112342196265072</v>
       </c>
-      <c r="K29" s="36" t="n">
+      <c r="M29" s="36" t="n">
         <v>-0.8784888126367574</v>
       </c>
-      <c r="L29" s="36" t="n">
+      <c r="N29" s="36" t="n">
         <v>10.26164617421538</v>
       </c>
-      <c r="M29" s="36" t="n">
+      <c r="O29" s="36" t="n">
         <v>-27.60812540431094</v>
       </c>
     </row>
@@ -2404,21 +2662,27 @@
         <v>74.02255312421833</v>
       </c>
       <c r="H30" s="36" t="n">
+        <v>-75.06489368360847</v>
+      </c>
+      <c r="I30" s="36" t="n">
+        <v>43.83007525897273</v>
+      </c>
+      <c r="J30" s="36" t="n">
         <v>16.86741300233976</v>
       </c>
-      <c r="I30" s="36" t="n">
+      <c r="K30" s="36" t="n">
         <v>30.47048112207599</v>
       </c>
-      <c r="J30" s="36" t="n">
+      <c r="L30" s="36" t="n">
         <v>38.16138272512508</v>
       </c>
-      <c r="K30" s="36" t="n">
+      <c r="M30" s="36" t="n">
         <v>287.2967731425879</v>
       </c>
-      <c r="L30" s="36" t="n">
+      <c r="N30" s="36" t="n">
         <v>302.2339379492017</v>
       </c>
-      <c r="M30" s="36" t="n">
+      <c r="O30" s="36" t="n">
         <v>28.42557524014479</v>
       </c>
     </row>
@@ -2442,21 +2706,27 @@
         <v>-18.28344971079963</v>
       </c>
       <c r="H31" s="36" t="n">
+        <v>-98.51333964406142</v>
+      </c>
+      <c r="I31" s="36" t="n">
+        <v>-55.28539610812211</v>
+      </c>
+      <c r="J31" s="36" t="n">
         <v>-59.19051592153274</v>
       </c>
-      <c r="I31" s="36" t="n">
+      <c r="K31" s="36" t="n">
         <v>-21.29304385919226</v>
       </c>
-      <c r="J31" s="36" t="n">
+      <c r="L31" s="36" t="n">
         <v>-25.97569354914944</v>
       </c>
-      <c r="K31" s="36" t="n">
+      <c r="M31" s="36" t="n">
         <v>-39.77301491739329</v>
       </c>
-      <c r="L31" s="36" t="n">
+      <c r="N31" s="36" t="n">
         <v>-49.46436623376201</v>
       </c>
-      <c r="M31" s="36" t="n">
+      <c r="O31" s="36" t="n">
         <v>-89.29024039042346</v>
       </c>
     </row>
@@ -2480,21 +2750,27 @@
         <v>0.5227490108479224</v>
       </c>
       <c r="H32" s="36" t="n">
+        <v>-45.57745532773993</v>
+      </c>
+      <c r="I32" s="36" t="n">
+        <v>-0.279321085990561</v>
+      </c>
+      <c r="J32" s="36" t="n">
         <v>-18.99021780684458</v>
       </c>
-      <c r="I32" s="36" t="n">
+      <c r="K32" s="36" t="n">
         <v>-2.537533620295328</v>
       </c>
-      <c r="J32" s="36" t="n">
+      <c r="L32" s="36" t="n">
         <v>-11.14424605903915</v>
       </c>
-      <c r="K32" s="36" t="n">
+      <c r="M32" s="36" t="n">
         <v>-12.62222792220395</v>
       </c>
-      <c r="L32" s="36" t="n">
+      <c r="N32" s="36" t="n">
         <v>-11.57372790097145</v>
       </c>
-      <c r="M32" s="36" t="n">
+      <c r="O32" s="36" t="n">
         <v>-30.32969491948224</v>
       </c>
     </row>
@@ -2518,21 +2794,27 @@
         <v>-6.562652756210437</v>
       </c>
       <c r="H33" s="36" t="n">
+        <v>13.76915497380155</v>
+      </c>
+      <c r="I33" s="36" t="n">
+        <v>-11.84137203749766</v>
+      </c>
+      <c r="J33" s="36" t="n">
         <v>36.0089755172143</v>
       </c>
-      <c r="I33" s="36" t="n">
+      <c r="K33" s="36" t="n">
         <v>19.77031354103625</v>
       </c>
-      <c r="J33" s="36" t="n">
+      <c r="L33" s="36" t="n">
         <v>3.953968438876255</v>
       </c>
-      <c r="K33" s="36" t="n">
+      <c r="M33" s="36" t="n">
         <v>79.68850259254869</v>
       </c>
-      <c r="L33" s="36" t="n">
+      <c r="N33" s="36" t="n">
         <v>64.01061290597922</v>
       </c>
-      <c r="M33" s="36" t="n">
+      <c r="O33" s="36" t="n">
         <v>29.66053238570699</v>
       </c>
     </row>
@@ -2556,21 +2838,27 @@
         <v>28.70951507435355</v>
       </c>
       <c r="H34" s="36" t="n">
+        <v>-99.50859422739981</v>
+      </c>
+      <c r="I34" s="36" t="n">
+        <v>-82.80214129231692</v>
+      </c>
+      <c r="J34" s="36" t="n">
         <v>-4.997019889193404</v>
       </c>
-      <c r="I34" s="36" t="n">
+      <c r="K34" s="36" t="n">
         <v>16.12559926399367</v>
       </c>
-      <c r="J34" s="36" t="n">
+      <c r="L34" s="36" t="n">
         <v>-2.363134911400063</v>
       </c>
-      <c r="K34" s="36" t="n">
+      <c r="M34" s="36" t="n">
         <v>-32.08848757684746</v>
       </c>
-      <c r="L34" s="36" t="n">
+      <c r="N34" s="36" t="n">
         <v>-49.98004143407833</v>
       </c>
-      <c r="M34" s="36" t="n">
+      <c r="O34" s="36" t="n">
         <v>-93.15490268073647</v>
       </c>
     </row>
@@ -2594,21 +2882,27 @@
         <v>-33.24624369916566</v>
       </c>
       <c r="H35" s="36" t="n">
+        <v>-75.85962318932157</v>
+      </c>
+      <c r="I35" s="36" t="n">
+        <v>-16.16831989920743</v>
+      </c>
+      <c r="J35" s="36" t="n">
         <v>-68.67022443453018</v>
       </c>
-      <c r="I35" s="36" t="n">
+      <c r="K35" s="36" t="n">
         <v>6.494124224558738</v>
       </c>
-      <c r="J35" s="36" t="n">
+      <c r="L35" s="36" t="n">
         <v>21.64890994872704</v>
       </c>
-      <c r="K35" s="36" t="n">
+      <c r="M35" s="36" t="n">
         <v>-9.278406194550849</v>
       </c>
-      <c r="L35" s="36" t="n">
+      <c r="N35" s="36" t="n">
         <v>-28.7872922618918</v>
       </c>
-      <c r="M35" s="36" t="n">
+      <c r="O35" s="36" t="n">
         <v>-67.06469903889177</v>
       </c>
     </row>
@@ -2632,21 +2926,27 @@
         <v>17.04974516602368</v>
       </c>
       <c r="H36" s="36" t="n">
+        <v>-94.61429300242932</v>
+      </c>
+      <c r="I36" s="36" t="n">
+        <v>-47.98572638006258</v>
+      </c>
+      <c r="J36" s="36" t="n">
         <v>-19.93647357626845</v>
       </c>
-      <c r="I36" s="36" t="n">
+      <c r="K36" s="36" t="n">
         <v>-29.15276075355244</v>
       </c>
-      <c r="J36" s="36" t="n">
+      <c r="L36" s="36" t="n">
         <v>-28.23724773382954</v>
       </c>
-      <c r="K36" s="36" t="n">
+      <c r="M36" s="36" t="n">
         <v>151.3807296338282</v>
       </c>
-      <c r="L36" s="36" t="n">
+      <c r="N36" s="36" t="n">
         <v>153.9805111283955</v>
       </c>
-      <c r="M36" s="36" t="n">
+      <c r="O36" s="36" t="n">
         <v>-39.72507210579246</v>
       </c>
     </row>
@@ -2670,21 +2970,27 @@
         <v>-12.16656389197989</v>
       </c>
       <c r="H37" s="36" t="n">
+        <v>-19.04136300395139</v>
+      </c>
+      <c r="I37" s="36" t="n">
+        <v>12.78506524074188</v>
+      </c>
+      <c r="J37" s="36" t="n">
         <v>-16.34719388822131</v>
       </c>
-      <c r="I37" s="36" t="n">
+      <c r="K37" s="36" t="n">
         <v>-20.24795733903337</v>
       </c>
-      <c r="J37" s="36" t="n">
+      <c r="L37" s="36" t="n">
         <v>-7.964830863080678</v>
       </c>
-      <c r="K37" s="36" t="n">
+      <c r="M37" s="36" t="n">
         <v>39.70331403261365</v>
       </c>
-      <c r="L37" s="36" t="n">
+      <c r="N37" s="36" t="n">
         <v>51.00831478187148</v>
       </c>
-      <c r="M37" s="36" t="n">
+      <c r="O37" s="36" t="n">
         <v>15.25374478868761</v>
       </c>
     </row>
@@ -2708,21 +3014,27 @@
         <v>-6.234333377151083</v>
       </c>
       <c r="H38" s="36" t="n">
+        <v>-21.882382398651</v>
+      </c>
+      <c r="I38" s="36" t="n">
+        <v>-1.156611158723273</v>
+      </c>
+      <c r="J38" s="36" t="n">
         <v>11.18383211438456</v>
       </c>
-      <c r="I38" s="36" t="n">
+      <c r="K38" s="36" t="n">
         <v>-16.19507129483321</v>
       </c>
-      <c r="J38" s="36" t="n">
+      <c r="L38" s="36" t="n">
         <v>-19.39275368388551</v>
       </c>
-      <c r="K38" s="36" t="n">
+      <c r="M38" s="36" t="n">
         <v>5.991671224850357</v>
       </c>
-      <c r="L38" s="36" t="n">
+      <c r="N38" s="36" t="n">
         <v>13.74697088203026</v>
       </c>
-      <c r="M38" s="36" t="n">
+      <c r="O38" s="36" t="n">
         <v>-0.1287247463308719</v>
       </c>
     </row>
@@ -2746,21 +3058,27 @@
         <v>-8.151625850031591</v>
       </c>
       <c r="H39" s="36" t="n">
+        <v>25.28283786477227</v>
+      </c>
+      <c r="I39" s="36" t="n">
+        <v>-2.39801342869288</v>
+      </c>
+      <c r="J39" s="36" t="n">
         <v>14.93847236504531</v>
       </c>
-      <c r="I39" s="36" t="n">
+      <c r="K39" s="36" t="n">
         <v>-11.00207497618331</v>
       </c>
-      <c r="J39" s="36" t="n">
+      <c r="L39" s="36" t="n">
         <v>-14.79740527516338</v>
       </c>
-      <c r="K39" s="36" t="n">
+      <c r="M39" s="36" t="n">
         <v>-18.71621865310299</v>
       </c>
-      <c r="L39" s="36" t="n">
+      <c r="N39" s="36" t="n">
         <v>-18.19724360934532</v>
       </c>
-      <c r="M39" s="36" t="n">
+      <c r="O39" s="36" t="n">
         <v>22.3088443108071</v>
       </c>
     </row>
@@ -2784,21 +3102,27 @@
         <v>-0.1408218127160009</v>
       </c>
       <c r="H40" s="36" t="n">
+        <v>-30.36540593054321</v>
+      </c>
+      <c r="I40" s="36" t="n">
+        <v>-0.3352767151336061</v>
+      </c>
+      <c r="J40" s="36" t="n">
         <v>4.8628835812243</v>
       </c>
-      <c r="I40" s="36" t="n">
+      <c r="K40" s="36" t="n">
         <v>51.03439884264372</v>
       </c>
-      <c r="J40" s="36" t="n">
+      <c r="L40" s="36" t="n">
         <v>37.63888402156968</v>
       </c>
-      <c r="K40" s="36" t="n">
+      <c r="M40" s="36" t="n">
         <v>25.59262130163343</v>
       </c>
-      <c r="L40" s="36" t="n">
+      <c r="N40" s="36" t="n">
         <v>2.74225772382814</v>
       </c>
-      <c r="M40" s="36" t="n">
+      <c r="O40" s="36" t="n">
         <v>-25.86714786813397</v>
       </c>
     </row>
@@ -2822,21 +3146,27 @@
         <v>-50.29851021472956</v>
       </c>
       <c r="H41" s="36" t="n">
+        <v>-65.99524141432394</v>
+      </c>
+      <c r="I41" s="36" t="n">
+        <v>-49.96333317261667</v>
+      </c>
+      <c r="J41" s="36" t="n">
         <v>-43.11442897485597</v>
       </c>
-      <c r="I41" s="36" t="n">
+      <c r="K41" s="36" t="n">
         <v>-58.87235427225367</v>
       </c>
-      <c r="J41" s="36" t="n">
+      <c r="L41" s="36" t="n">
         <v>-60.62578242722036</v>
       </c>
-      <c r="K41" s="36" t="n">
+      <c r="M41" s="36" t="n">
         <v>-14.2908372887692</v>
       </c>
-      <c r="L41" s="36" t="n">
+      <c r="N41" s="36" t="n">
         <v>-2.565594505845556</v>
       </c>
-      <c r="M41" s="36" t="n">
+      <c r="O41" s="36" t="n">
         <v>-38.63919591561025</v>
       </c>
     </row>
@@ -4107,7 +4437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -4123,14 +4453,14 @@
     <row r="2">
       <c r="A2" s="44" t="inlineStr">
         <is>
-          <t>Gerada/atualizada em 15/10/2026 por Scripts/gerar_planilha_comparacao.py a partir de: eventos_processados_manuais.xlsx, comparacao_volumes_medido_vs_calculado.csv,</t>
+          <t>Gerada/atualizada em 15/10/2026 (modelo adotado trocado em 26/10/2026) por Scripts/gerar_planilha_comparacao.py a partir de: eventos_processados_manuais.xlsx, comparacao_volumes_medido_vs_calculado.csv,</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>comparacao_qpico_convolucao_medido_vs_calculado.csv, comparacao_SY_previsao_vs_restrito.csv e comparacao_SY_modelo_com_base.csv (modelo com vazão de base).</t>
+          <t>comparacao_qpico_convolucao_medido_vs_calculado.csv, comparacao_SY_previsao_vs_restrito.csv, comparacao_SY_modelo_com_base.csv (vazão de base, não adotado) e comparacao_SY_so_direto.csv (adotado).</t>
         </is>
       </c>
     </row>
@@ -4168,71 +4498,85 @@
     <row r="9">
       <c r="A9" s="44" t="inlineStr">
         <is>
-          <t>• ADOTADO (15/10/2026): Q = escoamento direto (SCS-CN, λ = 0,20) + lâmina de vazão de base prevista, uniforme (kb·Qb_inicio·duração). Compara-se com a carga TOTAL medida.</t>
+          <t>• ADOTADO (26/10/2026): só escoamento direto, sem termo de vazão de base. Calculado: Q do SCS-CN (λ = 0,20); forçado: Q reescalado para o escoamento direto medido. Compara-se com a carga TOTAL medida (todo o sedimento do evento é atribuído ao escoamento superficial).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="44" t="inlineStr">
         <is>
-          <t>• Sem MUSLE: modelos triviais (SY proporcional ao volume ou à chuva), com um parâmetro c. Servem de régua: um modelo espacializado só se justifica se superar isso.</t>
+          <t>• Nesta planilha todas as escalas c são ajustadas por mínimos quadrados lineares; no texto do TCC a calibração adotada é em log (ver TCC_Texto/tabelas/).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="44" t="inlineStr">
         <is>
+          <t>• Não adotado (15 a 26/10/2026): Q = escoamento direto + lâmina de vazão de base prevista, uniforme (kb·Qb_inicio·duração). Removido: a vazão de base não produz erosão nas encostas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="44" t="inlineStr">
+        <is>
+          <t>• Sem MUSLE: modelos triviais (SY proporcional ao volume ou à chuva), com um parâmetro c. Servem de régua: um modelo espacializado só se justifica se superar isso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="44" t="inlineStr">
+        <is>
           <t>• α e β livres e FCI/DSC são experimentos que não foram adotados (valores só in-sample).</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="44" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="43" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="44" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="43" t="inlineStr">
         <is>
           <t>Pontos de atenção</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="44" t="inlineStr">
-        <is>
-          <t>• T_R_m3 (volume 'medido') = soma das vazões horárias × 3600: é o volume TOTAL, inclui a vazão de base (34–55%). SYY_t é a carga total (Q·CSS). O SCS-CN calcula só escoamento direto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="44" t="inlineStr">
-        <is>
-          <t>• NSE in-sample é otimista; o leave-one-out (c, e no modelo adotado também kb, refeitos sem o evento testado) é o valor honesto. Para α/β livres e FCI/DSC não foi calculado.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="44" t="inlineStr">
         <is>
-          <t>• O evento 15 responde por 49% da variância do SY medido; veja a coluna 'NSE sem o evento 15'. Com n = 17, os intervalos são largos (bootstrap do NSE do modelo adotado: [−0,96; 0,88]).</t>
+          <t>• T_R_m3 (volume 'medido') = soma das vazões horárias × 3600: é o volume TOTAL, inclui a vazão de base (34–55%). SYY_t é a carga total (Q·CSS). O SCS-CN calcula só escoamento direto.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="44" t="inlineStr">
         <is>
-          <t>• 'Q forçado', 'D e qp medidos' e os modelos 'Sem MUSLE' usam dado medido do evento; não são previsões puras e não devem ser comparados diretamente com a previsão de Hao et al. (2022).</t>
+          <t>• NSE in-sample é otimista; o leave-one-out (c, e no modelo adotado também kb, refeitos sem o evento testado) é o valor honesto. Para α/β livres e FCI/DSC não foi calculado.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="44" t="inlineStr">
         <is>
-          <t>• No modelo adotado, a duração é a janela observada do evento, kb é ajustado nos mesmos 17 eventos e λ foi fixado em 0,20 (padrão) depois de ver diagnósticos com outros valores.</t>
+          <t>• O evento 15 responde por 49% da variância do SY medido; veja a coluna 'NSE sem o evento 15'. Com n = 17, os intervalos são largos (bootstrap do NSE do modelo adotado: [−0,96; 0,88]).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>• 'Q forçado', 'D e qp medidos' e os modelos 'Sem MUSLE' usam dado medido do evento; não são previsões puras e não devem ser comparados diretamente com a previsão de Hao et al. (2022).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="44" t="inlineStr">
+        <is>
+          <t>• No modelo adotado, a duração é a janela observada do evento, kb é ajustado nos mesmos 17 eventos e λ foi fixado em 0,20 (padrão) depois de ver diagnósticos com outros valores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="44" t="inlineStr">
         <is>
           <t>• Os valores por evento de α/β livres e de FCI/DSC vêm das saídas de calibrar_alfa_beta_pixel.py (17/09) e da recalibração com a Eq. 8 exata (02/10); o FCI/DSC está arredondado em t.</t>
         </is>

</xml_diff>

<commit_message>
Regenera tabelas, figuras, mapas e planilha com o modelo oficial (CN-I, lambda 0,05, Woodward)
- Tabelas, figuras, mapas, fluxograma, escada do gargalo, Apendice B e planilha
  comparativa refeitos com o modelo oficial; tabela nova do evento 11 passo a passo
- Relatorio da regeneracao e anotacoes para declarar no texto (evento 17, erro
  absoluto do volume, nomes dos modelos)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Comparacao_Modelos_TCC.xlsx
+++ b/Comparacao_Modelos_TCC.xlsx
@@ -598,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -966,7 +966,7 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>ADOTADO — Espacializada — calculado: Q = só escoamento direto do SCS-CN (λ = 0,20)</t>
+          <t>ADOTADO (oficial, 28/10/2026) — Espacializada — MC: SCS-CN com CN-I, λ = 0,05 e S convertido (Woodward)</t>
         </is>
       </c>
       <c r="B10" s="14" t="n">
@@ -983,42 +983,42 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.01465768957838539</v>
+        <v>0.01535610579729387</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>-0.1430610598761948</v>
+        <v>0.1935679902313329</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>-1.111271232572765</v>
+        <v>-0.0978660470742716</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>0.8076337504346727</v>
+        <v>0.847441986652395</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-43.53950662539768</v>
+        <v>-30.14329035488577</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>-56.01578682027758</v>
+        <v>-35.72760719971373</v>
       </c>
       <c r="K10" s="17" t="n">
-        <v>60.61013891893332</v>
+        <v>46.1315226269715</v>
       </c>
       <c r="L10" s="16" t="n">
-        <v>-0.7833807874705723</v>
+        <v>-0.3984100229975116</v>
       </c>
       <c r="M10" s="16" t="n">
-        <v>-7.681737055638786</v>
+        <v>-1.48727062866628</v>
       </c>
       <c r="N10" s="13" t="inlineStr">
         <is>
-          <t>SY = c·ΣE_unit, com Q de cada pixel pelo SCS-CN (CN-I, λ = 0,20), sem termo de vazão de base (decisão de 26/10/2026). Aqui c por mínimos quadrados lineares, como nas demais linhas; no texto do TCC c é calibrado em log (tab_resultados.md).</t>
+          <t>SY = c*ΣE_unit, com Q de cada pixel pelo SCS-CN (CN-II da ANA convertido para CN-I; λ = 0,05; S0,05 = 25,4*1,33*(S0,20/25,4)^1,15, Woodward et al., 2003), sem termo de vazão de base. Aqui c por mínimos quadrados lineares, como nas demais linhas; no texto do TCC c é calibrado em log (tab_resultados.md).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>ADOTADO — Espacializada — forçado: Q reescalado para o escoamento direto medido</t>
+          <t>ADOTADO (oficial, 28/10/2026) — Espacializada — MFM: Q reescalado para o escoamento direto medido</t>
         </is>
       </c>
       <c r="B11" s="14" t="n">
@@ -1035,198 +1035,198 @@
         </is>
       </c>
       <c r="E11" s="15" t="n">
-        <v>0.02393903917940962</v>
+        <v>0.02256048706090509</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>0.8004067054076534</v>
+        <v>0.804010407155609</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>0.7878135588475967</v>
+        <v>0.7685167513635042</v>
       </c>
       <c r="H11" s="16" t="n">
-        <v>0.953407941825132</v>
+        <v>0.9473628845139359</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-7.441827102344136</v>
+        <v>-2.200636688367463</v>
       </c>
       <c r="J11" s="17" t="n">
-        <v>-10.93578435733297</v>
+        <v>6.302395669962201</v>
       </c>
       <c r="K11" s="17" t="n">
-        <v>28.33924567441559</v>
+        <v>24.89163759197071</v>
       </c>
       <c r="L11" s="16" t="n">
-        <v>0.5885851313896476</v>
+        <v>0.6236184573398615</v>
       </c>
       <c r="M11" s="16" t="n">
-        <v>0.4765633117073207</v>
+        <v>0.8555220664279796</v>
       </c>
       <c r="N11" s="13" t="inlineStr">
         <is>
-          <t>Q de cada pixel reescalado para o escoamento direto medido do evento (T_R − ΣBt·3600; limite Q ≤ chuva). Sem termo de base. Não é previsão: usa o volume medido. c por mínimos quadrados lineares nesta planilha.</t>
+          <t>Q de cada pixel (padrão do SCS-CN oficial) reescalado para o escoamento direto medido do evento (T_R - ΣBt*3600; limite Q ≤ chuva). Sem termo de base. Não é previsão: usa o volume medido. c por mínimos quadrados lineares nesta planilha.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
+          <t>Não adotado (26/10/2026) — Espacializada — calculado: só escoamento direto do SCS-CN (λ = 0,20)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>0.01465768957838539</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>-0.1430610598761948</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>-1.111271232572765</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>0.8076337504346727</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <v>-43.53950662539768</v>
+      </c>
+      <c r="J12" s="17" t="n">
+        <v>-56.01578682027758</v>
+      </c>
+      <c r="K12" s="17" t="n">
+        <v>60.61013891893332</v>
+      </c>
+      <c r="L12" s="16" t="n">
+        <v>-0.7833807874705723</v>
+      </c>
+      <c r="M12" s="16" t="n">
+        <v>-7.681737055638786</v>
+      </c>
+      <c r="N12" s="13" t="inlineStr">
+        <is>
+          <t>Modelo de 26/10/2026: SCS-CN com CN-I e λ = 0,20 (sem converter S), sem termo de vazão de base. Substituído pelo modelo oficial de 28/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Não adotado (26/10/2026) — Espacializada — forçado, padrão do SCS-CN com λ = 0,20</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Sim (volume direto)</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>0.02393903917940962</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>0.8004067054076534</v>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>0.7878135588475967</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>0.953407941825132</v>
+      </c>
+      <c r="I13" s="17" t="n">
+        <v>-7.441827102344136</v>
+      </c>
+      <c r="J13" s="17" t="n">
+        <v>-10.93578435733297</v>
+      </c>
+      <c r="K13" s="17" t="n">
+        <v>28.33924567441559</v>
+      </c>
+      <c r="L13" s="16" t="n">
+        <v>0.5885851313896476</v>
+      </c>
+      <c r="M13" s="16" t="n">
+        <v>0.4765633117073207</v>
+      </c>
+      <c r="N13" s="13" t="inlineStr">
+        <is>
+          <t>Modelo de 26/10/2026: Q reescalado para o escoamento direto medido, com o padrão espacial do SCS-CN com λ = 0,20. Substituído pelo modelo oficial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
           <t>Não adotado (até 26/10/2026) — Espacializada — Q = escoamento direto (λ = 0,20) + vazão de base prevista</t>
         </is>
       </c>
-      <c r="B12" s="14" t="n">
+      <c r="B14" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Parcial (Qb inicial e duração)</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E14" s="15" t="n">
         <v>0.01021554737345453</v>
       </c>
-      <c r="F12" s="16" t="n">
+      <c r="F14" s="16" t="n">
         <v>0.5014561479980195</v>
       </c>
-      <c r="G12" s="16" t="n">
+      <c r="G14" s="16" t="n">
         <v>0.3804165146048779</v>
       </c>
-      <c r="H12" s="16" t="n">
+      <c r="H14" s="16" t="n">
         <v>0.8926167512266159</v>
       </c>
-      <c r="I12" s="17" t="n">
+      <c r="I14" s="17" t="n">
         <v>-16.14184757409659</v>
       </c>
-      <c r="J12" s="17" t="n">
+      <c r="J14" s="17" t="n">
         <v>-12.08513115046434</v>
       </c>
-      <c r="K12" s="17" t="n">
+      <c r="K14" s="17" t="n">
         <v>28.47307387632832</v>
       </c>
-      <c r="L12" s="16" t="n">
+      <c r="L14" s="16" t="n">
         <v>0.07702056088139086</v>
       </c>
-      <c r="M12" s="16" t="n">
+      <c r="M14" s="16" t="n">
         <v>0.567804501948117</v>
       </c>
-      <c r="N12" s="13" t="inlineStr">
+      <c r="N14" s="13" t="inlineStr">
         <is>
           <t>Q do pixel = SCS-CN (CN-I, λ = 0,20) + lâmina de base uniforme = kb·Qb_inicio·duração (kb = 1,93). LOO aninhado (kb e c refeitos sem o evento). A duração é a da janela observada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Sem MUSLE — SY = c · volume total medido (T_R)</t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="19" t="inlineStr">
-        <is>
-          <t>Sim (volume)</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="n">
-        <v>0.0007961895562554518</v>
-      </c>
-      <c r="F13" s="21" t="n">
-        <v>0.8090940590219937</v>
-      </c>
-      <c r="G13" s="21" t="n">
-        <v>0.7653444578703972</v>
-      </c>
-      <c r="H13" s="21" t="n">
-        <v>0.9507257698920797</v>
-      </c>
-      <c r="I13" s="22" t="n">
-        <v>-3.391753649336037</v>
-      </c>
-      <c r="J13" s="22" t="n">
-        <v>-0.7984389704210787</v>
-      </c>
-      <c r="K13" s="22" t="n">
-        <v>19.10282680707302</v>
-      </c>
-      <c r="L13" s="21" t="n">
-        <v>0.6460347620386332</v>
-      </c>
-      <c r="M13" s="21" t="n">
-        <v>0.872949845816107</v>
-      </c>
-      <c r="N13" s="18" t="inlineStr">
-        <is>
-          <t>Referência trivial: sedimento proporcional ao volume total medido. Empata ou supera os modelos espacializados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Sem MUSLE — SY = c · escoamento direto medido</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>Sim (volume)</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E14" s="20" t="n">
-        <v>0.001498452605952412</v>
-      </c>
-      <c r="F14" s="21" t="n">
-        <v>0.7829694944221395</v>
-      </c>
-      <c r="G14" s="21" t="n">
-        <v>0.7326575009900256</v>
-      </c>
-      <c r="H14" s="21" t="n">
-        <v>0.944017090866361</v>
-      </c>
-      <c r="I14" s="22" t="n">
-        <v>-4.087214215008808</v>
-      </c>
-      <c r="J14" s="22" t="n">
-        <v>-1.378850569568219</v>
-      </c>
-      <c r="K14" s="22" t="n">
-        <v>20.40253847958454</v>
-      </c>
-      <c r="L14" s="21" t="n">
-        <v>0.623484423390292</v>
-      </c>
-      <c r="M14" s="21" t="n">
-        <v>0.8619387224365678</v>
-      </c>
-      <c r="N14" s="18" t="inlineStr">
-        <is>
-          <t>Mesma referência, com o escoamento direto (T_R − Σ Bt·3600).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>Sem MUSLE — SY = c · chuva do evento</t>
+          <t>Sem MUSLE — SY = c · volume total medido (T_R)</t>
         </is>
       </c>
       <c r="B15" s="19" t="n">
@@ -1234,188 +1234,292 @@
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
+          <t>Sim (volume)</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>0.0007961895562554518</v>
+      </c>
+      <c r="F15" s="21" t="n">
+        <v>0.8090940590219937</v>
+      </c>
+      <c r="G15" s="21" t="n">
+        <v>0.7653444578703972</v>
+      </c>
+      <c r="H15" s="21" t="n">
+        <v>0.9507257698920797</v>
+      </c>
+      <c r="I15" s="22" t="n">
+        <v>-3.391753649336037</v>
+      </c>
+      <c r="J15" s="22" t="n">
+        <v>-0.7984389704210787</v>
+      </c>
+      <c r="K15" s="22" t="n">
+        <v>19.10282680707302</v>
+      </c>
+      <c r="L15" s="21" t="n">
+        <v>0.6460347620386332</v>
+      </c>
+      <c r="M15" s="21" t="n">
+        <v>0.872949845816107</v>
+      </c>
+      <c r="N15" s="18" t="inlineStr">
+        <is>
+          <t>Referência trivial: sedimento proporcional ao volume total medido. Empata ou supera os modelos espacializados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Sem MUSLE — SY = c · escoamento direto medido</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Sim (volume)</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>0.001498452605952412</v>
+      </c>
+      <c r="F16" s="21" t="n">
+        <v>0.7829694944221395</v>
+      </c>
+      <c r="G16" s="21" t="n">
+        <v>0.7326575009900256</v>
+      </c>
+      <c r="H16" s="21" t="n">
+        <v>0.944017090866361</v>
+      </c>
+      <c r="I16" s="22" t="n">
+        <v>-4.087214215008808</v>
+      </c>
+      <c r="J16" s="22" t="n">
+        <v>-1.378850569568219</v>
+      </c>
+      <c r="K16" s="22" t="n">
+        <v>20.40253847958454</v>
+      </c>
+      <c r="L16" s="21" t="n">
+        <v>0.623484423390292</v>
+      </c>
+      <c r="M16" s="21" t="n">
+        <v>0.8619387224365678</v>
+      </c>
+      <c r="N16" s="18" t="inlineStr">
+        <is>
+          <t>Mesma referência, com o escoamento direto (T_R − Σ Bt·3600).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Sem MUSLE — SY = c · chuva do evento</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
           <t>Sim (chuva)</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E17" s="20" t="n">
         <v>22.32215182996425</v>
       </c>
-      <c r="F15" s="21" t="n">
+      <c r="F17" s="21" t="n">
         <v>0.670573753905237</v>
       </c>
-      <c r="G15" s="21" t="n">
+      <c r="G17" s="21" t="n">
         <v>0.6050248690021753</v>
       </c>
-      <c r="H15" s="21" t="n">
+      <c r="H17" s="21" t="n">
         <v>0.8930732205069412</v>
       </c>
-      <c r="I15" s="22" t="n">
+      <c r="I17" s="22" t="n">
         <v>0.3555526316416786</v>
       </c>
-      <c r="J15" s="22" t="n">
+      <c r="J17" s="22" t="n">
         <v>31.56009507155892</v>
       </c>
-      <c r="K15" s="22" t="n">
+      <c r="K17" s="22" t="n">
         <v>55.83818107257348</v>
       </c>
-      <c r="L15" s="21" t="n">
+      <c r="L17" s="21" t="n">
         <v>0.4322127199602186</v>
       </c>
-      <c r="M15" s="21" t="n">
+      <c r="M17" s="21" t="n">
         <v>0.5638685217717554</v>
       </c>
-      <c r="N15" s="18" t="inlineStr">
+      <c r="N17" s="18" t="inlineStr">
         <is>
           <t>Referência trivial: sedimento proporcional à lâmina de chuva do evento (não usa vazão).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="23" t="inlineStr">
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>Espacializada — α e β livres (experimento, não adotado)</t>
         </is>
       </c>
-      <c r="B16" s="24" t="n">
+      <c r="B18" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="C16" s="24" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="D16" s="24" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="E16" s="24" t="n"/>
-      <c r="F16" s="25" t="n">
+      <c r="E18" s="24" t="n"/>
+      <c r="F18" s="25" t="n">
         <v>0.6120927741732798</v>
       </c>
-      <c r="G16" s="24" t="inlineStr">
+      <c r="G18" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H16" s="25" t="n">
+      <c r="H18" s="25" t="n">
         <v>0.8779670710651121</v>
       </c>
-      <c r="I16" s="26" t="n">
+      <c r="I18" s="26" t="n">
         <v>-1.359787660971752</v>
       </c>
-      <c r="J16" s="26" t="n">
+      <c r="J18" s="26" t="n">
         <v>29.23856688755154</v>
       </c>
-      <c r="K16" s="26" t="n">
+      <c r="K18" s="26" t="n">
         <v>57.85399063634824</v>
       </c>
-      <c r="L16" s="25" t="n">
+      <c r="L18" s="25" t="n">
         <v>0.2794748944469283</v>
       </c>
-      <c r="M16" s="25" t="n">
+      <c r="M18" s="25" t="n">
         <v>0.5037305280139199</v>
       </c>
-      <c r="N16" s="23" t="inlineStr">
+      <c r="N18" s="23" t="inlineStr">
         <is>
           <t>α = 4,22 e β = 0,28 ajustados na fórmula por pixel (NSE bruto). Só in-sample; instável em eventos pequenos.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="23" t="inlineStr">
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>Espacializada — com FCI/DSC de Hao (descartado)</t>
         </is>
       </c>
-      <c r="B17" s="24" t="n">
+      <c r="B19" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="D17" s="24" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="E17" s="24" t="n"/>
-      <c r="F17" s="25" t="n">
+      <c r="E19" s="24" t="n"/>
+      <c r="F19" s="25" t="n">
         <v>0.2059722483388605</v>
       </c>
-      <c r="G17" s="24" t="inlineStr">
+      <c r="G19" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H17" s="25" t="n">
+      <c r="H19" s="25" t="n">
         <v>0.8492652457985379</v>
       </c>
-      <c r="I17" s="26" t="n">
+      <c r="I19" s="26" t="n">
         <v>-27.60542986665604</v>
       </c>
-      <c r="J17" s="26" t="n">
+      <c r="J19" s="26" t="n">
         <v>-30.81712256272602</v>
       </c>
-      <c r="K17" s="26" t="n">
+      <c r="K19" s="26" t="n">
         <v>46.47290066656894</v>
       </c>
-      <c r="L17" s="25" t="n">
+      <c r="L19" s="25" t="n">
         <v>-0.5201467513534836</v>
       </c>
-      <c r="M17" s="25" t="n">
+      <c r="M19" s="25" t="n">
         <v>-1.100415318018777</v>
       </c>
-      <c r="N17" s="23" t="inlineStr">
+      <c r="N19" s="23" t="inlineStr">
         <is>
           <t>Eq. 8 exata, objetivo NSE bruto: FCI₀ = 3,17 (limite da busca) e k = 4,90. Só in-sample; valores por evento arredondados.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="27" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>Legenda de cores</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="28" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
         <is>
           <t>Referência</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="29" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>Concentrada (um D e um qp por evento)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="30" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
         <is>
           <t>Espacializada (pixel a pixel)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="31" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t>Referência sem MUSLE (modelo trivial)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="32" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t>Experimento não adotado</t>
         </is>
@@ -1435,7 +1539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1453,6 +1557,8 @@
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1500,40 +1606,50 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>ADOTADO — Espacializada — calculado: Q = só escoamento direto do SCS-CN (λ = 0,20)</t>
+          <t>ADOTADO (oficial, 28/10/2026) — Espacializada — MC: SCS-CN com CN-I, λ = 0,05 e S convertido (Woodward)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>ADOTADO — Espacializada — forçado: Q reescalado para o escoamento direto medido</t>
+          <t>ADOTADO (oficial, 28/10/2026) — Espacializada — MFM: Q reescalado para o escoamento direto medido</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
+          <t>Não adotado (26/10/2026) — Espacializada — calculado: só escoamento direto do SCS-CN (λ = 0,20)</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Não adotado (26/10/2026) — Espacializada — forçado, padrão do SCS-CN com λ = 0,20</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
           <t>Não adotado (até 26/10/2026) — Espacializada — Q = escoamento direto (λ = 0,20) + vazão de base prevista</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · volume total medido (T_R)</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · escoamento direto medido</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · chuva do evento</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Espacializada — α e β livres (experimento, não adotado)</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>Espacializada — com FCI/DSC de Hao (descartado)</t>
         </is>
@@ -1562,27 +1678,33 @@
         <v>449.3170466927465</v>
       </c>
       <c r="H4" s="35" t="n">
+        <v>33.1907545444036</v>
+      </c>
+      <c r="I4" s="35" t="n">
+        <v>363.0003163154691</v>
+      </c>
+      <c r="J4" s="35" t="n">
         <v>3.395812369796301</v>
       </c>
-      <c r="I4" s="35" t="n">
+      <c r="K4" s="35" t="n">
         <v>112.1412828113571</v>
       </c>
-      <c r="J4" s="35" t="n">
+      <c r="L4" s="35" t="n">
         <v>345.3114725244459</v>
       </c>
-      <c r="K4" s="35" t="n">
+      <c r="M4" s="35" t="n">
         <v>325.6612740094749</v>
       </c>
-      <c r="L4" s="35" t="n">
+      <c r="N4" s="35" t="n">
         <v>335.3462273397419</v>
       </c>
-      <c r="M4" s="35" t="n">
+      <c r="O4" s="35" t="n">
         <v>521.5406672974292</v>
       </c>
-      <c r="N4" s="35" t="n">
+      <c r="P4" s="35" t="n">
         <v>402.31</v>
       </c>
-      <c r="O4" s="35" t="n">
+      <c r="Q4" s="35" t="n">
         <v>44</v>
       </c>
     </row>
@@ -1609,27 +1731,33 @@
         <v>1952.709995741231</v>
       </c>
       <c r="H5" s="35" t="n">
+        <v>442.1812384248472</v>
+      </c>
+      <c r="I5" s="35" t="n">
+        <v>2474.838031800356</v>
+      </c>
+      <c r="J5" s="35" t="n">
         <v>221.9471536947734</v>
       </c>
-      <c r="I5" s="35" t="n">
+      <c r="K5" s="35" t="n">
         <v>2446.152720547311</v>
       </c>
-      <c r="J5" s="35" t="n">
+      <c r="L5" s="35" t="n">
         <v>556.7738625138491</v>
       </c>
-      <c r="K5" s="35" t="n">
+      <c r="M5" s="35" t="n">
         <v>2093.89095210065</v>
       </c>
-      <c r="L5" s="35" t="n">
+      <c r="N5" s="35" t="n">
         <v>2594.041412751792</v>
       </c>
-      <c r="M5" s="35" t="n">
+      <c r="O5" s="35" t="n">
         <v>1279.94063140894</v>
       </c>
-      <c r="N5" s="35" t="n">
+      <c r="P5" s="35" t="n">
         <v>1166.06</v>
       </c>
-      <c r="O5" s="35" t="n">
+      <c r="Q5" s="35" t="n">
         <v>458</v>
       </c>
     </row>
@@ -1656,27 +1784,33 @@
         <v>1217.715307419696</v>
       </c>
       <c r="H6" s="35" t="n">
+        <v>1141.490583101922</v>
+      </c>
+      <c r="I6" s="35" t="n">
+        <v>1268.440754136698</v>
+      </c>
+      <c r="J6" s="35" t="n">
         <v>715.2497859025611</v>
       </c>
-      <c r="I6" s="35" t="n">
+      <c r="K6" s="35" t="n">
         <v>1345.46939045668</v>
       </c>
-      <c r="J6" s="35" t="n">
+      <c r="L6" s="35" t="n">
         <v>1110.545019820355</v>
       </c>
-      <c r="K6" s="35" t="n">
+      <c r="M6" s="35" t="n">
         <v>852.1056303154498</v>
       </c>
-      <c r="L6" s="35" t="n">
+      <c r="N6" s="35" t="n">
         <v>876.4850816002048</v>
       </c>
-      <c r="M6" s="35" t="n">
+      <c r="O6" s="35" t="n">
         <v>1460.56347873917</v>
       </c>
-      <c r="N6" s="35" t="n">
+      <c r="P6" s="35" t="n">
         <v>1774.47</v>
       </c>
-      <c r="O6" s="35" t="n">
+      <c r="Q6" s="35" t="n">
         <v>1275</v>
       </c>
     </row>
@@ -1703,27 +1837,33 @@
         <v>2105.91594721014</v>
       </c>
       <c r="H7" s="35" t="n">
+        <v>189.2495409120935</v>
+      </c>
+      <c r="I7" s="35" t="n">
+        <v>2179.725776669924</v>
+      </c>
+      <c r="J7" s="35" t="n">
         <v>45.54912984079175</v>
       </c>
-      <c r="I7" s="35" t="n">
+      <c r="K7" s="35" t="n">
         <v>1273.278586203443</v>
       </c>
-      <c r="J7" s="35" t="n">
+      <c r="L7" s="35" t="n">
         <v>816.9741376043581</v>
       </c>
-      <c r="K7" s="35" t="n">
+      <c r="M7" s="35" t="n">
         <v>1356.35062941391</v>
       </c>
-      <c r="L7" s="35" t="n">
+      <c r="N7" s="35" t="n">
         <v>1479.638590906746</v>
       </c>
-      <c r="M7" s="35" t="n">
+      <c r="O7" s="35" t="n">
         <v>807.7466937250238</v>
       </c>
-      <c r="N7" s="35" t="n">
+      <c r="P7" s="35" t="n">
         <v>830.3200000000001</v>
       </c>
-      <c r="O7" s="35" t="n">
+      <c r="Q7" s="35" t="n">
         <v>219</v>
       </c>
     </row>
@@ -1750,27 +1890,33 @@
         <v>1937.226684229344</v>
       </c>
       <c r="H8" s="35" t="n">
+        <v>908.6661108368021</v>
+      </c>
+      <c r="I8" s="35" t="n">
+        <v>1633.860608533617</v>
+      </c>
+      <c r="J8" s="35" t="n">
         <v>583.6999398535477</v>
       </c>
-      <c r="I8" s="35" t="n">
+      <c r="K8" s="35" t="n">
         <v>1733.516766331042</v>
       </c>
-      <c r="J8" s="35" t="n">
+      <c r="L8" s="35" t="n">
         <v>1455.288174287584</v>
       </c>
-      <c r="K8" s="35" t="n">
+      <c r="M8" s="35" t="n">
         <v>1464.698970511554</v>
       </c>
-      <c r="L8" s="35" t="n">
+      <c r="N8" s="35" t="n">
         <v>1246.70682591335</v>
       </c>
-      <c r="M8" s="35" t="n">
+      <c r="O8" s="35" t="n">
         <v>1359.650667409476</v>
       </c>
-      <c r="N8" s="35" t="n">
+      <c r="P8" s="35" t="n">
         <v>1512.46</v>
       </c>
-      <c r="O8" s="35" t="n">
+      <c r="Q8" s="35" t="n">
         <v>993</v>
       </c>
     </row>
@@ -1797,27 +1943,33 @@
         <v>345.5367123230465</v>
       </c>
       <c r="H9" s="35" t="n">
+        <v>206.8419928576781</v>
+      </c>
+      <c r="I9" s="35" t="n">
+        <v>357.7227326212673</v>
+      </c>
+      <c r="J9" s="35" t="n">
         <v>49.51079330413807</v>
       </c>
-      <c r="I9" s="35" t="n">
+      <c r="K9" s="35" t="n">
         <v>285.5869566669709</v>
       </c>
-      <c r="J9" s="35" t="n">
+      <c r="L9" s="35" t="n">
         <v>232.0502770563494</v>
       </c>
-      <c r="K9" s="35" t="n">
+      <c r="M9" s="35" t="n">
         <v>259.0603361045289</v>
       </c>
-      <c r="L9" s="35" t="n">
+      <c r="N9" s="35" t="n">
         <v>274.3312812033558</v>
       </c>
-      <c r="M9" s="35" t="n">
+      <c r="O9" s="35" t="n">
         <v>769.0109774995045</v>
       </c>
-      <c r="N9" s="35" t="n">
+      <c r="P9" s="35" t="n">
         <v>798.67</v>
       </c>
-      <c r="O9" s="35" t="n">
+      <c r="Q9" s="35" t="n">
         <v>255</v>
       </c>
     </row>
@@ -1844,27 +1996,33 @@
         <v>1075.844277632001</v>
       </c>
       <c r="H10" s="35" t="n">
+        <v>120.118574695528</v>
+      </c>
+      <c r="I10" s="35" t="n">
+        <v>954.112180316272</v>
+      </c>
+      <c r="J10" s="35" t="n">
         <v>19.57271851367251</v>
       </c>
-      <c r="I10" s="35" t="n">
+      <c r="K10" s="35" t="n">
         <v>588.6928725381608</v>
       </c>
-      <c r="J10" s="35" t="n">
+      <c r="L10" s="35" t="n">
         <v>537.2797770286651</v>
       </c>
-      <c r="K10" s="35" t="n">
+      <c r="M10" s="35" t="n">
         <v>1036.221280441298</v>
       </c>
-      <c r="L10" s="35" t="n">
+      <c r="N10" s="35" t="n">
         <v>974.5715674362018</v>
       </c>
-      <c r="M10" s="35" t="n">
+      <c r="O10" s="35" t="n">
         <v>792.9220828686108</v>
       </c>
-      <c r="N10" s="35" t="n">
+      <c r="P10" s="35" t="n">
         <v>665.33</v>
       </c>
-      <c r="O10" s="35" t="n">
+      <c r="Q10" s="35" t="n">
         <v>141</v>
       </c>
     </row>
@@ -1891,27 +2049,33 @@
         <v>2119.52449650215</v>
       </c>
       <c r="H11" s="35" t="n">
+        <v>1430.245945359113</v>
+      </c>
+      <c r="I11" s="35" t="n">
+        <v>1950.346786058603</v>
+      </c>
+      <c r="J11" s="35" t="n">
         <v>1147.500617819254</v>
       </c>
-      <c r="I11" s="35" t="n">
+      <c r="K11" s="35" t="n">
         <v>2102.61282989047</v>
       </c>
-      <c r="J11" s="35" t="n">
+      <c r="L11" s="35" t="n">
         <v>1708.093138162858</v>
       </c>
-      <c r="K11" s="35" t="n">
+      <c r="M11" s="35" t="n">
         <v>2054.998366180861</v>
       </c>
-      <c r="L11" s="35" t="n">
+      <c r="N11" s="35" t="n">
         <v>1873.525634607447</v>
       </c>
-      <c r="M11" s="35" t="n">
+      <c r="O11" s="35" t="n">
         <v>1842.362352711668</v>
       </c>
-      <c r="N11" s="35" t="n">
+      <c r="P11" s="35" t="n">
         <v>1864.47</v>
       </c>
-      <c r="O11" s="35" t="n">
+      <c r="Q11" s="35" t="n">
         <v>1469</v>
       </c>
     </row>
@@ -1938,27 +2102,33 @@
         <v>1078.784008134861</v>
       </c>
       <c r="H12" s="35" t="n">
+        <v>1516.949623043454</v>
+      </c>
+      <c r="I12" s="35" t="n">
+        <v>943.6956329801276</v>
+      </c>
+      <c r="J12" s="35" t="n">
         <v>1313.525572216108</v>
       </c>
-      <c r="I12" s="35" t="n">
+      <c r="K12" s="35" t="n">
         <v>1017.838378661586</v>
       </c>
-      <c r="J12" s="35" t="n">
+      <c r="L12" s="35" t="n">
         <v>1570.296161854369</v>
       </c>
-      <c r="K12" s="35" t="n">
+      <c r="M12" s="35" t="n">
         <v>1382.812148553971</v>
       </c>
-      <c r="L12" s="35" t="n">
+      <c r="N12" s="35" t="n">
         <v>1200.204008804088</v>
       </c>
-      <c r="M12" s="35" t="n">
+      <c r="O12" s="35" t="n">
         <v>2074.59959813259</v>
       </c>
-      <c r="N12" s="35" t="n">
+      <c r="P12" s="35" t="n">
         <v>1893.59</v>
       </c>
-      <c r="O12" s="35" t="n">
+      <c r="Q12" s="35" t="n">
         <v>1497</v>
       </c>
     </row>
@@ -1985,27 +2155,33 @@
         <v>1090.583745727621</v>
       </c>
       <c r="H13" s="35" t="n">
+        <v>44.85413196582799</v>
+      </c>
+      <c r="I13" s="35" t="n">
+        <v>797.6101976112188</v>
+      </c>
+      <c r="J13" s="35" t="n">
         <v>4.1637881072344</v>
       </c>
-      <c r="I13" s="35" t="n">
+      <c r="K13" s="35" t="n">
         <v>145.7212013974608</v>
       </c>
-      <c r="J13" s="35" t="n">
+      <c r="L13" s="35" t="n">
         <v>804.9809359057639</v>
       </c>
-      <c r="K13" s="35" t="n">
+      <c r="M13" s="35" t="n">
         <v>983.9574871137551</v>
       </c>
-      <c r="L13" s="35" t="n">
+      <c r="N13" s="35" t="n">
         <v>827.2984168102502</v>
       </c>
-      <c r="M13" s="35" t="n">
+      <c r="O13" s="35" t="n">
         <v>575.4290314409496</v>
       </c>
-      <c r="N13" s="35" t="n">
+      <c r="P13" s="35" t="n">
         <v>423.83</v>
       </c>
-      <c r="O13" s="35" t="n">
+      <c r="Q13" s="35" t="n">
         <v>58</v>
       </c>
     </row>
@@ -2032,27 +2208,33 @@
         <v>1216.088895856651</v>
       </c>
       <c r="H14" s="35" t="n">
+        <v>627.8281160515097</v>
+      </c>
+      <c r="I14" s="35" t="n">
+        <v>1431.482924547073</v>
+      </c>
+      <c r="J14" s="35" t="n">
         <v>439.7781609316646</v>
       </c>
-      <c r="I14" s="35" t="n">
+      <c r="K14" s="35" t="n">
         <v>1527.206571449622</v>
       </c>
-      <c r="J14" s="35" t="n">
+      <c r="L14" s="35" t="n">
         <v>570.7512848138058</v>
       </c>
-      <c r="K14" s="35" t="n">
+      <c r="M14" s="35" t="n">
         <v>1940.060441839825</v>
       </c>
-      <c r="L14" s="35" t="n">
+      <c r="N14" s="35" t="n">
         <v>2216.143282110158</v>
       </c>
-      <c r="M14" s="35" t="n">
+      <c r="O14" s="35" t="n">
         <v>1652.72381593072</v>
       </c>
-      <c r="N14" s="35" t="n">
+      <c r="P14" s="35" t="n">
         <v>1297.32</v>
       </c>
-      <c r="O14" s="35" t="n">
+      <c r="Q14" s="35" t="n">
         <v>600</v>
       </c>
     </row>
@@ -2079,27 +2261,33 @@
         <v>246.6252247066325</v>
       </c>
       <c r="H15" s="35" t="n">
+        <v>91.45453541121327</v>
+      </c>
+      <c r="I15" s="35" t="n">
+        <v>229.154750482815</v>
+      </c>
+      <c r="J15" s="35" t="n">
         <v>11.3477495965152</v>
       </c>
-      <c r="I15" s="35" t="n">
+      <c r="K15" s="35" t="n">
         <v>109.5947018190772</v>
       </c>
-      <c r="J15" s="35" t="n">
+      <c r="L15" s="35" t="n">
         <v>168.6948157559068</v>
       </c>
-      <c r="K15" s="35" t="n">
+      <c r="M15" s="35" t="n">
         <v>149.2759875232221</v>
       </c>
-      <c r="L15" s="35" t="n">
+      <c r="N15" s="35" t="n">
         <v>151.2049844970366</v>
       </c>
-      <c r="M15" s="35" t="n">
+      <c r="O15" s="35" t="n">
         <v>529.6622290370957</v>
       </c>
-      <c r="N15" s="35" t="n">
+      <c r="P15" s="35" t="n">
         <v>535.14</v>
       </c>
-      <c r="O15" s="35" t="n">
+      <c r="Q15" s="35" t="n">
         <v>127</v>
       </c>
     </row>
@@ -2126,27 +2314,33 @@
         <v>1050.918637090984</v>
       </c>
       <c r="H16" s="35" t="n">
+        <v>1303.815210975021</v>
+      </c>
+      <c r="I16" s="35" t="n">
+        <v>1254.255894587459</v>
+      </c>
+      <c r="J16" s="35" t="n">
         <v>968.6623252219821</v>
       </c>
-      <c r="I16" s="35" t="n">
+      <c r="K16" s="35" t="n">
         <v>1349.462486031505</v>
       </c>
-      <c r="J16" s="35" t="n">
+      <c r="L16" s="35" t="n">
         <v>1000.897800237597</v>
       </c>
-      <c r="K16" s="35" t="n">
+      <c r="M16" s="35" t="n">
         <v>954.225539752419</v>
       </c>
-      <c r="L16" s="35" t="n">
+      <c r="N16" s="35" t="n">
         <v>1101.191969705689</v>
       </c>
-      <c r="M16" s="35" t="n">
+      <c r="O16" s="35" t="n">
         <v>1671.536750534142</v>
       </c>
-      <c r="N16" s="35" t="n">
+      <c r="P16" s="35" t="n">
         <v>1806.8</v>
       </c>
-      <c r="O16" s="35" t="n">
+      <c r="Q16" s="35" t="n">
         <v>1379</v>
       </c>
     </row>
@@ -2173,27 +2367,33 @@
         <v>1623.297962092956</v>
       </c>
       <c r="H17" s="35" t="n">
+        <v>1653.628145168578</v>
+      </c>
+      <c r="I17" s="35" t="n">
+        <v>1586.385888716231</v>
+      </c>
+      <c r="J17" s="35" t="n">
         <v>1352.394474684254</v>
       </c>
-      <c r="I17" s="35" t="n">
+      <c r="K17" s="35" t="n">
         <v>1711.20493728039</v>
       </c>
-      <c r="J17" s="35" t="n">
+      <c r="L17" s="35" t="n">
         <v>1924.84621065964</v>
       </c>
-      <c r="K17" s="35" t="n">
+      <c r="M17" s="35" t="n">
         <v>1450.854826507385</v>
       </c>
-      <c r="L17" s="35" t="n">
+      <c r="N17" s="35" t="n">
         <v>1395.495637024438</v>
       </c>
-      <c r="M17" s="35" t="n">
+      <c r="O17" s="35" t="n">
         <v>1834.958040560652</v>
       </c>
-      <c r="N17" s="35" t="n">
+      <c r="P17" s="35" t="n">
         <v>1969.22</v>
       </c>
-      <c r="O17" s="35" t="n">
+      <c r="Q17" s="35" t="n">
         <v>1729</v>
       </c>
     </row>
@@ -2220,27 +2420,33 @@
         <v>3516.719813419875</v>
       </c>
       <c r="H18" s="35" t="n">
+        <v>4627.830496287419</v>
+      </c>
+      <c r="I18" s="35" t="n">
+        <v>3475.558739133969</v>
+      </c>
+      <c r="J18" s="35" t="n">
         <v>4796.869212743336</v>
       </c>
-      <c r="I18" s="35" t="n">
+      <c r="K18" s="35" t="n">
         <v>3737.015958976279</v>
       </c>
-      <c r="J18" s="35" t="n">
+      <c r="L18" s="35" t="n">
         <v>4400.800850653997</v>
       </c>
-      <c r="K18" s="35" t="n">
+      <c r="M18" s="35" t="n">
         <v>3407.580909091359</v>
       </c>
-      <c r="L18" s="35" t="n">
+      <c r="N18" s="35" t="n">
         <v>3262.264093367402</v>
       </c>
-      <c r="M18" s="35" t="n">
+      <c r="O18" s="35" t="n">
         <v>3112.21931817309</v>
       </c>
-      <c r="N18" s="35" t="n">
+      <c r="P18" s="35" t="n">
         <v>3132.09</v>
       </c>
-      <c r="O18" s="35" t="n">
+      <c r="Q18" s="35" t="n">
         <v>4683</v>
       </c>
     </row>
@@ -2267,27 +2473,33 @@
         <v>1733.627651320199</v>
       </c>
       <c r="H19" s="35" t="n">
+        <v>1356.152259655845</v>
+      </c>
+      <c r="I19" s="35" t="n">
+        <v>1604.742736526617</v>
+      </c>
+      <c r="J19" s="35" t="n">
         <v>1208.906982399343</v>
       </c>
-      <c r="I19" s="35" t="n">
+      <c r="K19" s="35" t="n">
         <v>1730.251773390043</v>
       </c>
-      <c r="J19" s="35" t="n">
+      <c r="L19" s="35" t="n">
         <v>1820.495600641051</v>
       </c>
-      <c r="K19" s="35" t="n">
+      <c r="M19" s="35" t="n">
         <v>2622.066542977747</v>
       </c>
-      <c r="L19" s="35" t="n">
+      <c r="N19" s="35" t="n">
         <v>2389.51070465581</v>
       </c>
-      <c r="M19" s="35" t="n">
+      <c r="O19" s="35" t="n">
         <v>2180.37885993762</v>
       </c>
-      <c r="N19" s="35" t="n">
+      <c r="P19" s="35" t="n">
         <v>1783.68</v>
       </c>
-      <c r="O19" s="35" t="n">
+      <c r="Q19" s="35" t="n">
         <v>1287</v>
       </c>
     </row>
@@ -2314,27 +2526,33 @@
         <v>849.6769813029938</v>
       </c>
       <c r="H20" s="35" t="n">
+        <v>963.3318621799533</v>
+      </c>
+      <c r="I20" s="35" t="n">
+        <v>816.0196196375981</v>
+      </c>
+      <c r="J20" s="35" t="n">
         <v>581.3318826023811</v>
       </c>
-      <c r="I20" s="35" t="n">
+      <c r="K20" s="35" t="n">
         <v>855.4070352425226</v>
       </c>
-      <c r="J20" s="35" t="n">
+      <c r="L20" s="35" t="n">
         <v>972.4931883765348</v>
       </c>
-      <c r="K20" s="35" t="n">
+      <c r="M20" s="35" t="n">
         <v>703.101939620467</v>
       </c>
-      <c r="L20" s="35" t="n">
+      <c r="N20" s="35" t="n">
         <v>673.1260264621188</v>
       </c>
-      <c r="M20" s="35" t="n">
+      <c r="O20" s="35" t="n">
         <v>1465.24989405988</v>
       </c>
-      <c r="N20" s="35" t="n">
+      <c r="P20" s="35" t="n">
         <v>1665.7</v>
       </c>
-      <c r="O20" s="35" t="n">
+      <c r="Q20" s="35" t="n">
         <v>1049</v>
       </c>
     </row>
@@ -2383,40 +2601,50 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>ADOTADO — Espacializada — calculado: Q = só escoamento direto do SCS-CN (λ = 0,20)</t>
+          <t>ADOTADO (oficial, 28/10/2026) — Espacializada — MC: SCS-CN com CN-I, λ = 0,05 e S convertido (Woodward)</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>ADOTADO — Espacializada — forçado: Q reescalado para o escoamento direto medido</t>
+          <t>ADOTADO (oficial, 28/10/2026) — Espacializada — MFM: Q reescalado para o escoamento direto medido</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
+          <t>Não adotado (26/10/2026) — Espacializada — calculado: só escoamento direto do SCS-CN (λ = 0,20)</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Não adotado (26/10/2026) — Espacializada — forçado, padrão do SCS-CN com λ = 0,20</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
           <t>Não adotado (até 26/10/2026) — Espacializada — Q = escoamento direto (λ = 0,20) + vazão de base prevista</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · volume total medido (T_R)</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · escoamento direto medido</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="O24" s="3" t="inlineStr">
         <is>
           <t>Sem MUSLE — SY = c · chuva do evento</t>
         </is>
       </c>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="P24" s="3" t="inlineStr">
         <is>
           <t>Espacializada — α e β livres (experimento, não adotado)</t>
         </is>
       </c>
-      <c r="O24" s="3" t="inlineStr">
+      <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>Espacializada — com FCI/DSC de Hao (descartado)</t>
         </is>
@@ -2442,27 +2670,33 @@
         <v>68.69003876798844</v>
       </c>
       <c r="H25" s="36" t="n">
+        <v>-87.53897785083831</v>
+      </c>
+      <c r="I25" s="36" t="n">
+        <v>36.28358390311006</v>
+      </c>
+      <c r="J25" s="36" t="n">
         <v>-98.72508794285413</v>
       </c>
-      <c r="I25" s="36" t="n">
+      <c r="K25" s="36" t="n">
         <v>-57.89806444206479</v>
       </c>
-      <c r="J25" s="36" t="n">
+      <c r="L25" s="36" t="n">
         <v>29.64254553870305</v>
       </c>
-      <c r="K25" s="36" t="n">
+      <c r="M25" s="36" t="n">
         <v>22.26514293693651</v>
       </c>
-      <c r="L25" s="36" t="n">
+      <c r="N25" s="36" t="n">
         <v>25.90122833537476</v>
       </c>
-      <c r="M25" s="36" t="n">
+      <c r="O25" s="36" t="n">
         <v>95.8054252182597</v>
       </c>
-      <c r="N25" s="36" t="n">
+      <c r="P25" s="36" t="n">
         <v>51.04187565613901</v>
       </c>
-      <c r="O25" s="36" t="n">
+      <c r="Q25" s="36" t="n">
         <v>-83.48079210342742</v>
       </c>
     </row>
@@ -2486,27 +2720,33 @@
         <v>-4.27354939043077</v>
       </c>
       <c r="H26" s="36" t="n">
+        <v>-78.32323254714186</v>
+      </c>
+      <c r="I26" s="36" t="n">
+        <v>21.32239868413866</v>
+      </c>
+      <c r="J26" s="36" t="n">
         <v>-89.11962693260433</v>
       </c>
-      <c r="I26" s="36" t="n">
+      <c r="K26" s="36" t="n">
         <v>19.91617705528769</v>
       </c>
-      <c r="J26" s="36" t="n">
+      <c r="L26" s="36" t="n">
         <v>-72.70563178000242</v>
       </c>
-      <c r="K26" s="36" t="n">
+      <c r="M26" s="36" t="n">
         <v>2.647474148869351</v>
       </c>
-      <c r="L26" s="36" t="n">
+      <c r="N26" s="36" t="n">
         <v>27.16602962986431</v>
       </c>
-      <c r="M26" s="36" t="n">
+      <c r="O26" s="36" t="n">
         <v>-37.25429075337954</v>
       </c>
-      <c r="N26" s="36" t="n">
+      <c r="P26" s="36" t="n">
         <v>-42.83698795968764</v>
       </c>
-      <c r="O26" s="36" t="n">
+      <c r="Q26" s="36" t="n">
         <v>-77.54775953684796</v>
       </c>
     </row>
@@ -2530,27 +2770,33 @@
         <v>31.25100713804224</v>
       </c>
       <c r="H27" s="36" t="n">
+        <v>23.03515259916248</v>
+      </c>
+      <c r="I27" s="36" t="n">
+        <v>36.71843119731699</v>
+      </c>
+      <c r="J27" s="36" t="n">
         <v>-22.90705866718269</v>
       </c>
-      <c r="I27" s="36" t="n">
+      <c r="K27" s="36" t="n">
         <v>45.02093510267608</v>
       </c>
-      <c r="J27" s="36" t="n">
+      <c r="L27" s="36" t="n">
         <v>19.6996961731722</v>
       </c>
-      <c r="K27" s="36" t="n">
+      <c r="M27" s="36" t="n">
         <v>-8.156100621019334</v>
       </c>
-      <c r="L27" s="36" t="n">
+      <c r="N27" s="36" t="n">
         <v>-5.528370218765239</v>
       </c>
-      <c r="M27" s="36" t="n">
+      <c r="O27" s="36" t="n">
         <v>57.42631007880354</v>
       </c>
-      <c r="N27" s="36" t="n">
+      <c r="P27" s="36" t="n">
         <v>91.26061175148753</v>
       </c>
-      <c r="O27" s="36" t="n">
+      <c r="Q27" s="36" t="n">
         <v>37.4254171573183</v>
       </c>
     </row>
@@ -2574,27 +2820,33 @@
         <v>52.6179140483064</v>
       </c>
       <c r="H28" s="36" t="n">
+        <v>-86.28488938180722</v>
+      </c>
+      <c r="I28" s="36" t="n">
+        <v>57.96698898329447</v>
+      </c>
+      <c r="J28" s="36" t="n">
         <v>-96.69900729313228</v>
       </c>
-      <c r="I28" s="36" t="n">
+      <c r="K28" s="36" t="n">
         <v>-7.724179549434214</v>
       </c>
-      <c r="J28" s="36" t="n">
+      <c r="L28" s="36" t="n">
         <v>-40.79303645628863</v>
       </c>
-      <c r="K28" s="36" t="n">
+      <c r="M28" s="36" t="n">
         <v>-1.703862372336926</v>
       </c>
-      <c r="L28" s="36" t="n">
+      <c r="N28" s="36" t="n">
         <v>7.230944135601576</v>
       </c>
-      <c r="M28" s="36" t="n">
+      <c r="O28" s="36" t="n">
         <v>-41.46175888973972</v>
       </c>
-      <c r="N28" s="36" t="n">
+      <c r="P28" s="36" t="n">
         <v>-39.82584795918982</v>
       </c>
-      <c r="O28" s="36" t="n">
+      <c r="Q28" s="36" t="n">
         <v>-84.12884273901938</v>
       </c>
     </row>
@@ -2618,27 +2870,33 @@
         <v>41.22806766178572</v>
       </c>
       <c r="H29" s="36" t="n">
+        <v>-33.75625060921423</v>
+      </c>
+      <c r="I29" s="36" t="n">
+        <v>19.11201639456376</v>
+      </c>
+      <c r="J29" s="36" t="n">
         <v>-57.44699612548916</v>
       </c>
-      <c r="I29" s="36" t="n">
+      <c r="K29" s="36" t="n">
         <v>26.37716853752386</v>
       </c>
-      <c r="J29" s="36" t="n">
+      <c r="L29" s="36" t="n">
         <v>6.093694877760371</v>
       </c>
-      <c r="K29" s="36" t="n">
+      <c r="M29" s="36" t="n">
         <v>6.779762531427293</v>
       </c>
-      <c r="L29" s="36" t="n">
+      <c r="N29" s="36" t="n">
         <v>-9.112342196265072</v>
       </c>
-      <c r="M29" s="36" t="n">
+      <c r="O29" s="36" t="n">
         <v>-0.8784888126367574</v>
       </c>
-      <c r="N29" s="36" t="n">
+      <c r="P29" s="36" t="n">
         <v>10.26164617421538</v>
       </c>
-      <c r="O29" s="36" t="n">
+      <c r="Q29" s="36" t="n">
         <v>-27.60812540431094</v>
       </c>
     </row>
@@ -2662,27 +2920,33 @@
         <v>74.02255312421833</v>
       </c>
       <c r="H30" s="36" t="n">
+        <v>4.171772221824431</v>
+      </c>
+      <c r="I30" s="36" t="n">
+        <v>80.15979495436375</v>
+      </c>
+      <c r="J30" s="36" t="n">
         <v>-75.06489368360847</v>
       </c>
-      <c r="I30" s="36" t="n">
+      <c r="K30" s="36" t="n">
         <v>43.83007525897273</v>
       </c>
-      <c r="J30" s="36" t="n">
+      <c r="L30" s="36" t="n">
         <v>16.86741300233976</v>
       </c>
-      <c r="K30" s="36" t="n">
+      <c r="M30" s="36" t="n">
         <v>30.47048112207599</v>
       </c>
-      <c r="L30" s="36" t="n">
+      <c r="N30" s="36" t="n">
         <v>38.16138272512508</v>
       </c>
-      <c r="M30" s="36" t="n">
+      <c r="O30" s="36" t="n">
         <v>287.2967731425879</v>
       </c>
-      <c r="N30" s="36" t="n">
+      <c r="P30" s="36" t="n">
         <v>302.2339379492017</v>
       </c>
-      <c r="O30" s="36" t="n">
+      <c r="Q30" s="36" t="n">
         <v>28.42557524014479</v>
       </c>
     </row>
@@ -2706,27 +2970,33 @@
         <v>-18.28344971079963</v>
       </c>
       <c r="H31" s="36" t="n">
+        <v>-90.87630454160235</v>
+      </c>
+      <c r="I31" s="36" t="n">
+        <v>-27.52970147690629</v>
+      </c>
+      <c r="J31" s="36" t="n">
         <v>-98.51333964406142</v>
       </c>
-      <c r="I31" s="36" t="n">
+      <c r="K31" s="36" t="n">
         <v>-55.28539610812211</v>
       </c>
-      <c r="J31" s="36" t="n">
+      <c r="L31" s="36" t="n">
         <v>-59.19051592153274</v>
       </c>
-      <c r="K31" s="36" t="n">
+      <c r="M31" s="36" t="n">
         <v>-21.29304385919226</v>
       </c>
-      <c r="L31" s="36" t="n">
+      <c r="N31" s="36" t="n">
         <v>-25.97569354914944</v>
       </c>
-      <c r="M31" s="36" t="n">
+      <c r="O31" s="36" t="n">
         <v>-39.77301491739329</v>
       </c>
-      <c r="N31" s="36" t="n">
+      <c r="P31" s="36" t="n">
         <v>-49.46436623376201</v>
       </c>
-      <c r="O31" s="36" t="n">
+      <c r="Q31" s="36" t="n">
         <v>-89.29024039042346</v>
       </c>
     </row>
@@ -2750,27 +3020,33 @@
         <v>0.5227490108479224</v>
       </c>
       <c r="H32" s="36" t="n">
+        <v>-32.16768457907219</v>
+      </c>
+      <c r="I32" s="36" t="n">
+        <v>-7.500847108570325</v>
+      </c>
+      <c r="J32" s="36" t="n">
         <v>-45.57745532773993</v>
       </c>
-      <c r="I32" s="36" t="n">
+      <c r="K32" s="36" t="n">
         <v>-0.279321085990561</v>
       </c>
-      <c r="J32" s="36" t="n">
+      <c r="L32" s="36" t="n">
         <v>-18.99021780684458</v>
       </c>
-      <c r="K32" s="36" t="n">
+      <c r="M32" s="36" t="n">
         <v>-2.537533620295328</v>
       </c>
-      <c r="L32" s="36" t="n">
+      <c r="N32" s="36" t="n">
         <v>-11.14424605903915</v>
       </c>
-      <c r="M32" s="36" t="n">
+      <c r="O32" s="36" t="n">
         <v>-12.62222792220395</v>
       </c>
-      <c r="N32" s="36" t="n">
+      <c r="P32" s="36" t="n">
         <v>-11.57372790097145</v>
       </c>
-      <c r="O32" s="36" t="n">
+      <c r="Q32" s="36" t="n">
         <v>-30.32969491948224</v>
       </c>
     </row>
@@ -2794,27 +3070,33 @@
         <v>-6.562652756210437</v>
       </c>
       <c r="H33" s="36" t="n">
+        <v>31.38844069880549</v>
+      </c>
+      <c r="I33" s="36" t="n">
+        <v>-18.26314082680689</v>
+      </c>
+      <c r="J33" s="36" t="n">
         <v>13.76915497380155</v>
       </c>
-      <c r="I33" s="36" t="n">
+      <c r="K33" s="36" t="n">
         <v>-11.84137203749766</v>
       </c>
-      <c r="J33" s="36" t="n">
+      <c r="L33" s="36" t="n">
         <v>36.0089755172143</v>
       </c>
-      <c r="K33" s="36" t="n">
+      <c r="M33" s="36" t="n">
         <v>19.77031354103625</v>
       </c>
-      <c r="L33" s="36" t="n">
+      <c r="N33" s="36" t="n">
         <v>3.953968438876255</v>
       </c>
-      <c r="M33" s="36" t="n">
+      <c r="O33" s="36" t="n">
         <v>79.68850259254869</v>
       </c>
-      <c r="N33" s="36" t="n">
+      <c r="P33" s="36" t="n">
         <v>64.01061290597922</v>
       </c>
-      <c r="O33" s="36" t="n">
+      <c r="Q33" s="36" t="n">
         <v>29.66053238570699</v>
       </c>
     </row>
@@ -2838,27 +3120,33 @@
         <v>28.70951507435355</v>
       </c>
       <c r="H34" s="36" t="n">
+        <v>-94.70636381935896</v>
+      </c>
+      <c r="I34" s="36" t="n">
+        <v>-5.866906457141392</v>
+      </c>
+      <c r="J34" s="36" t="n">
         <v>-99.50859422739981</v>
       </c>
-      <c r="I34" s="36" t="n">
+      <c r="K34" s="36" t="n">
         <v>-82.80214129231692</v>
       </c>
-      <c r="J34" s="36" t="n">
+      <c r="L34" s="36" t="n">
         <v>-4.997019889193404</v>
       </c>
-      <c r="K34" s="36" t="n">
+      <c r="M34" s="36" t="n">
         <v>16.12559926399367</v>
       </c>
-      <c r="L34" s="36" t="n">
+      <c r="N34" s="36" t="n">
         <v>-2.363134911400063</v>
       </c>
-      <c r="M34" s="36" t="n">
+      <c r="O34" s="36" t="n">
         <v>-32.08848757684746</v>
       </c>
-      <c r="N34" s="36" t="n">
+      <c r="P34" s="36" t="n">
         <v>-49.98004143407833</v>
       </c>
-      <c r="O34" s="36" t="n">
+      <c r="Q34" s="36" t="n">
         <v>-93.15490268073647</v>
       </c>
     </row>
@@ -2882,27 +3170,33 @@
         <v>-33.24624369916566</v>
       </c>
       <c r="H35" s="36" t="n">
+        <v>-65.53715340999658</v>
+      </c>
+      <c r="I35" s="36" t="n">
+        <v>-21.42279843225796</v>
+      </c>
+      <c r="J35" s="36" t="n">
         <v>-75.85962318932157</v>
       </c>
-      <c r="I35" s="36" t="n">
+      <c r="K35" s="36" t="n">
         <v>-16.16831989920743</v>
       </c>
-      <c r="J35" s="36" t="n">
+      <c r="L35" s="36" t="n">
         <v>-68.67022443453018</v>
       </c>
-      <c r="K35" s="36" t="n">
+      <c r="M35" s="36" t="n">
         <v>6.494124224558738</v>
       </c>
-      <c r="L35" s="36" t="n">
+      <c r="N35" s="36" t="n">
         <v>21.64890994872704</v>
       </c>
-      <c r="M35" s="36" t="n">
+      <c r="O35" s="36" t="n">
         <v>-9.278406194550849</v>
       </c>
-      <c r="N35" s="36" t="n">
+      <c r="P35" s="36" t="n">
         <v>-28.7872922618918</v>
       </c>
-      <c r="O35" s="36" t="n">
+      <c r="Q35" s="36" t="n">
         <v>-67.06469903889177</v>
       </c>
     </row>
@@ -2926,27 +3220,33 @@
         <v>17.04974516602368</v>
       </c>
       <c r="H36" s="36" t="n">
+        <v>-56.59515332669976</v>
+      </c>
+      <c r="I36" s="36" t="n">
+        <v>8.758157968242491</v>
+      </c>
+      <c r="J36" s="36" t="n">
         <v>-94.61429300242932</v>
       </c>
-      <c r="I36" s="36" t="n">
+      <c r="K36" s="36" t="n">
         <v>-47.98572638006258</v>
       </c>
-      <c r="J36" s="36" t="n">
+      <c r="L36" s="36" t="n">
         <v>-19.93647357626845</v>
       </c>
-      <c r="K36" s="36" t="n">
+      <c r="M36" s="36" t="n">
         <v>-29.15276075355244</v>
       </c>
-      <c r="L36" s="36" t="n">
+      <c r="N36" s="36" t="n">
         <v>-28.23724773382954</v>
       </c>
-      <c r="M36" s="36" t="n">
+      <c r="O36" s="36" t="n">
         <v>151.3807296338282</v>
       </c>
-      <c r="N36" s="36" t="n">
+      <c r="P36" s="36" t="n">
         <v>153.9805111283955</v>
       </c>
-      <c r="O36" s="36" t="n">
+      <c r="Q36" s="36" t="n">
         <v>-39.72507210579246</v>
       </c>
     </row>
@@ -2970,27 +3270,33 @@
         <v>-12.16656389197989</v>
       </c>
       <c r="H37" s="36" t="n">
+        <v>8.969967786311816</v>
+      </c>
+      <c r="I37" s="36" t="n">
+        <v>4.827910641399606</v>
+      </c>
+      <c r="J37" s="36" t="n">
         <v>-19.04136300395139</v>
       </c>
-      <c r="I37" s="36" t="n">
+      <c r="K37" s="36" t="n">
         <v>12.78506524074188</v>
       </c>
-      <c r="J37" s="36" t="n">
+      <c r="L37" s="36" t="n">
         <v>-16.34719388822131</v>
       </c>
-      <c r="K37" s="36" t="n">
+      <c r="M37" s="36" t="n">
         <v>-20.24795733903337</v>
       </c>
-      <c r="L37" s="36" t="n">
+      <c r="N37" s="36" t="n">
         <v>-7.964830863080678</v>
       </c>
-      <c r="M37" s="36" t="n">
+      <c r="O37" s="36" t="n">
         <v>39.70331403261365</v>
       </c>
-      <c r="N37" s="36" t="n">
+      <c r="P37" s="36" t="n">
         <v>51.00831478187148</v>
       </c>
-      <c r="O37" s="36" t="n">
+      <c r="Q37" s="36" t="n">
         <v>15.25374478868761</v>
       </c>
     </row>
@@ -3014,27 +3320,33 @@
         <v>-6.234333377151083</v>
       </c>
       <c r="H38" s="36" t="n">
+        <v>-4.482387707723873</v>
+      </c>
+      <c r="I38" s="36" t="n">
+        <v>-8.366465152969781</v>
+      </c>
+      <c r="J38" s="36" t="n">
         <v>-21.882382398651</v>
       </c>
-      <c r="I38" s="36" t="n">
+      <c r="K38" s="36" t="n">
         <v>-1.156611158723273</v>
       </c>
-      <c r="J38" s="36" t="n">
+      <c r="L38" s="36" t="n">
         <v>11.18383211438456</v>
       </c>
-      <c r="K38" s="36" t="n">
+      <c r="M38" s="36" t="n">
         <v>-16.19507129483321</v>
       </c>
-      <c r="L38" s="36" t="n">
+      <c r="N38" s="36" t="n">
         <v>-19.39275368388551</v>
       </c>
-      <c r="M38" s="36" t="n">
+      <c r="O38" s="36" t="n">
         <v>5.991671224850357</v>
       </c>
-      <c r="N38" s="36" t="n">
+      <c r="P38" s="36" t="n">
         <v>13.74697088203026</v>
       </c>
-      <c r="O38" s="36" t="n">
+      <c r="Q38" s="36" t="n">
         <v>-0.1287247463308719</v>
       </c>
     </row>
@@ -3058,27 +3370,33 @@
         <v>-8.151625850031591</v>
       </c>
       <c r="H39" s="36" t="n">
+        <v>20.86794782558682</v>
+      </c>
+      <c r="I39" s="36" t="n">
+        <v>-9.226655409395331</v>
+      </c>
+      <c r="J39" s="36" t="n">
         <v>25.28283786477227</v>
       </c>
-      <c r="I39" s="36" t="n">
+      <c r="K39" s="36" t="n">
         <v>-2.39801342869288</v>
       </c>
-      <c r="J39" s="36" t="n">
+      <c r="L39" s="36" t="n">
         <v>14.93847236504531</v>
       </c>
-      <c r="K39" s="36" t="n">
+      <c r="M39" s="36" t="n">
         <v>-11.00207497618331</v>
       </c>
-      <c r="L39" s="36" t="n">
+      <c r="N39" s="36" t="n">
         <v>-14.79740527516338</v>
       </c>
-      <c r="M39" s="36" t="n">
+      <c r="O39" s="36" t="n">
         <v>-18.71621865310299</v>
       </c>
-      <c r="N39" s="36" t="n">
+      <c r="P39" s="36" t="n">
         <v>-18.19724360934532</v>
       </c>
-      <c r="O39" s="36" t="n">
+      <c r="Q39" s="36" t="n">
         <v>22.3088443108071</v>
       </c>
     </row>
@@ -3102,27 +3420,33 @@
         <v>-0.1408218127160009</v>
       </c>
       <c r="H40" s="36" t="n">
+        <v>-21.88388894066605</v>
+      </c>
+      <c r="I40" s="36" t="n">
+        <v>-7.564758355389445</v>
+      </c>
+      <c r="J40" s="36" t="n">
         <v>-30.36540593054321</v>
       </c>
-      <c r="I40" s="36" t="n">
+      <c r="K40" s="36" t="n">
         <v>-0.3352767151336061</v>
       </c>
-      <c r="J40" s="36" t="n">
+      <c r="L40" s="36" t="n">
         <v>4.8628835812243</v>
       </c>
-      <c r="K40" s="36" t="n">
+      <c r="M40" s="36" t="n">
         <v>51.03439884264372</v>
       </c>
-      <c r="L40" s="36" t="n">
+      <c r="N40" s="36" t="n">
         <v>37.63888402156968</v>
       </c>
-      <c r="M40" s="36" t="n">
+      <c r="O40" s="36" t="n">
         <v>25.59262130163343</v>
       </c>
-      <c r="N40" s="36" t="n">
+      <c r="P40" s="36" t="n">
         <v>2.74225772382814</v>
       </c>
-      <c r="O40" s="36" t="n">
+      <c r="Q40" s="36" t="n">
         <v>-25.86714786813397</v>
       </c>
     </row>
@@ -3146,27 +3470,33 @@
         <v>-50.29851021472956</v>
       </c>
       <c r="H41" s="36" t="n">
+        <v>-43.65031681270309</v>
+      </c>
+      <c r="I41" s="36" t="n">
+        <v>-52.26728311763498</v>
+      </c>
+      <c r="J41" s="36" t="n">
         <v>-65.99524141432394</v>
       </c>
-      <c r="I41" s="36" t="n">
+      <c r="K41" s="36" t="n">
         <v>-49.96333317261667</v>
       </c>
-      <c r="J41" s="36" t="n">
+      <c r="L41" s="36" t="n">
         <v>-43.11442897485597</v>
       </c>
-      <c r="K41" s="36" t="n">
+      <c r="M41" s="36" t="n">
         <v>-58.87235427225367</v>
       </c>
-      <c r="L41" s="36" t="n">
+      <c r="N41" s="36" t="n">
         <v>-60.62578242722036</v>
       </c>
-      <c r="M41" s="36" t="n">
+      <c r="O41" s="36" t="n">
         <v>-14.2908372887692</v>
       </c>
-      <c r="N41" s="36" t="n">
+      <c r="P41" s="36" t="n">
         <v>-2.565594505845556</v>
       </c>
-      <c r="O41" s="36" t="n">
+      <c r="Q41" s="36" t="n">
         <v>-38.63919591561025</v>
       </c>
     </row>
@@ -3181,7 +3511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:Z20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3205,6 +3535,11 @@
     <col width="16" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3320,6 +3655,31 @@
           <t>Erro do volume total previsto (%)</t>
         </is>
       </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Escoamento direto medido, oficial (m³)</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
+          <t>Escoamento direto SCS-CN oficial, λ = 0,05 com S convertido (m³)</t>
+        </is>
+      </c>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>SCS-CN oficial / medido</t>
+        </is>
+      </c>
+      <c r="Y3" s="3" t="inlineStr">
+        <is>
+          <t>ΣE_unit oficial, MC</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
+          <t>ΣE_unit oficial, MFM</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="34" t="n">
@@ -3385,6 +3745,21 @@
       <c r="U4" s="37" t="n">
         <v>-15.15502481408893</v>
       </c>
+      <c r="V4" s="40" t="n">
+        <v>223795.0176119162</v>
+      </c>
+      <c r="W4" s="40" t="n">
+        <v>35538.54167340556</v>
+      </c>
+      <c r="X4" s="41" t="n">
+        <v>0.1587995213326558</v>
+      </c>
+      <c r="Y4" s="40" t="n">
+        <v>2161.404393961172</v>
+      </c>
+      <c r="Z4" s="40" t="n">
+        <v>16090.09217467249</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="34" t="n">
@@ -3450,6 +3825,21 @@
       <c r="U5" s="37" t="n">
         <v>-64.32095723029425</v>
       </c>
+      <c r="V5" s="40" t="n">
+        <v>1731146.785989288</v>
+      </c>
+      <c r="W5" s="40" t="n">
+        <v>521004.9123078882</v>
+      </c>
+      <c r="X5" s="41" t="n">
+        <v>0.3009594082515381</v>
+      </c>
+      <c r="Y5" s="40" t="n">
+        <v>28795.14144157372</v>
+      </c>
+      <c r="Z5" s="40" t="n">
+        <v>109697.8990355658</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="34" t="n">
@@ -3515,6 +3905,21 @@
       <c r="U6" s="37" t="n">
         <v>1.966614643311005</v>
       </c>
+      <c r="V6" s="40" t="n">
+        <v>584926.7958949648</v>
+      </c>
+      <c r="W6" s="40" t="n">
+        <v>750546.9697405144</v>
+      </c>
+      <c r="X6" s="41" t="n">
+        <v>1.283146839925743</v>
+      </c>
+      <c r="Y6" s="40" t="n">
+        <v>74334.6391441951</v>
+      </c>
+      <c r="Z6" s="40" t="n">
+        <v>56223.99688058021</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="34" t="n">
@@ -3580,6 +3985,21 @@
       <c r="U7" s="37" t="n">
         <v>-54.46942401582405</v>
       </c>
+      <c r="V7" s="40" t="n">
+        <v>987444.370965802</v>
+      </c>
+      <c r="W7" s="40" t="n">
+        <v>154471.268763171</v>
+      </c>
+      <c r="X7" s="41" t="n">
+        <v>0.1564354137864854</v>
+      </c>
+      <c r="Y7" s="40" t="n">
+        <v>12324.05815707808</v>
+      </c>
+      <c r="Z7" s="40" t="n">
+        <v>96616.96446470587</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="34" t="n">
@@ -3645,6 +4065,21 @@
       <c r="U8" s="37" t="n">
         <v>-12.26790946159734</v>
       </c>
+      <c r="V8" s="40" t="n">
+        <v>831996.1678874366</v>
+      </c>
+      <c r="W8" s="40" t="n">
+        <v>694670.8864142008</v>
+      </c>
+      <c r="X8" s="41" t="n">
+        <v>0.8349448149239372</v>
+      </c>
+      <c r="Y8" s="40" t="n">
+        <v>59172.95197307978</v>
+      </c>
+      <c r="Z8" s="40" t="n">
+        <v>72421.33576827437</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="34" t="n">
@@ -3710,6 +4145,21 @@
       <c r="U9" s="37" t="n">
         <v>-15.19869864023432</v>
       </c>
+      <c r="V9" s="40" t="n">
+        <v>183076.3816710717</v>
+      </c>
+      <c r="W9" s="40" t="n">
+        <v>158263.9199523317</v>
+      </c>
+      <c r="X9" s="41" t="n">
+        <v>0.8644693461152193</v>
+      </c>
+      <c r="Y9" s="40" t="n">
+        <v>13469.69053144508</v>
+      </c>
+      <c r="Z9" s="40" t="n">
+        <v>15856.16177769328</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="34" t="n">
@@ -3775,6 +4225,21 @@
       <c r="U10" s="37" t="n">
         <v>-39.142622354315</v>
       </c>
+      <c r="V10" s="40" t="n">
+        <v>650385.3131989896</v>
+      </c>
+      <c r="W10" s="40" t="n">
+        <v>141725.3584473097</v>
+      </c>
+      <c r="X10" s="41" t="n">
+        <v>0.2179098383237137</v>
+      </c>
+      <c r="Y10" s="40" t="n">
+        <v>7822.202860616911</v>
+      </c>
+      <c r="Z10" s="40" t="n">
+        <v>42291.29352307496</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="34" t="n">
@@ -3840,6 +4305,21 @@
       <c r="U11" s="37" t="n">
         <v>-10.72623685629839</v>
       </c>
+      <c r="V11" s="40" t="n">
+        <v>1250306.901376196</v>
+      </c>
+      <c r="W11" s="40" t="n">
+        <v>1336334.180068558</v>
+      </c>
+      <c r="X11" s="41" t="n">
+        <v>1.068804929891751</v>
+      </c>
+      <c r="Y11" s="40" t="n">
+        <v>93138.58371639757</v>
+      </c>
+      <c r="Z11" s="40" t="n">
+        <v>86449.67552311161</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="34" t="n">
@@ -3905,6 +4385,21 @@
       <c r="U12" s="37" t="n">
         <v>50.92947459250861</v>
       </c>
+      <c r="V12" s="40" t="n">
+        <v>800962.2753742293</v>
+      </c>
+      <c r="W12" s="40" t="n">
+        <v>1725171.322891924</v>
+      </c>
+      <c r="X12" s="41" t="n">
+        <v>2.15387337947456</v>
+      </c>
+      <c r="Y12" s="40" t="n">
+        <v>98784.78587395372</v>
+      </c>
+      <c r="Z12" s="40" t="n">
+        <v>41829.57710232466</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="34" t="n">
@@ -3970,6 +4465,21 @@
       <c r="U13" s="37" t="n">
         <v>-12.52391152233077</v>
       </c>
+      <c r="V13" s="40" t="n">
+        <v>552101.8239241685</v>
+      </c>
+      <c r="W13" s="40" t="n">
+        <v>56645.16034796761</v>
+      </c>
+      <c r="X13" s="41" t="n">
+        <v>0.1025991183027641</v>
+      </c>
+      <c r="Y13" s="40" t="n">
+        <v>2920.931423494908</v>
+      </c>
+      <c r="Z13" s="40" t="n">
+        <v>35354.29866642338</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="34" t="n">
@@ -4035,6 +4545,21 @@
       <c r="U14" s="37" t="n">
         <v>-45.05556343597437</v>
       </c>
+      <c r="V14" s="40" t="n">
+        <v>1478954.538372993</v>
+      </c>
+      <c r="W14" s="40" t="n">
+        <v>997495.0961575384</v>
+      </c>
+      <c r="X14" s="41" t="n">
+        <v>0.6744596066183948</v>
+      </c>
+      <c r="Y14" s="40" t="n">
+        <v>40884.59172781609</v>
+      </c>
+      <c r="Z14" s="40" t="n">
+        <v>63450.88741579873</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="34" t="n">
@@ -4100,6 +4625,21 @@
       <c r="U15" s="37" t="n">
         <v>-13.23735916023795</v>
       </c>
+      <c r="V15" s="40" t="n">
+        <v>100907.4186907174</v>
+      </c>
+      <c r="W15" s="40" t="n">
+        <v>62527.37828872128</v>
+      </c>
+      <c r="X15" s="41" t="n">
+        <v>0.61965095431059</v>
+      </c>
+      <c r="Y15" s="40" t="n">
+        <v>5955.581227327169</v>
+      </c>
+      <c r="Z15" s="40" t="n">
+        <v>10157.34943417581</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="34" t="n">
@@ -4165,6 +4705,21 @@
       <c r="U16" s="37" t="n">
         <v>3.731718853166846</v>
       </c>
+      <c r="V16" s="40" t="n">
+        <v>734886.085373234</v>
+      </c>
+      <c r="W16" s="40" t="n">
+        <v>1072541.274636831</v>
+      </c>
+      <c r="X16" s="41" t="n">
+        <v>1.459466026074107</v>
+      </c>
+      <c r="Y16" s="40" t="n">
+        <v>84905.32874583256</v>
+      </c>
+      <c r="Z16" s="40" t="n">
+        <v>55595.24895014124</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="34" t="n">
@@ -4230,6 +4785,21 @@
       <c r="U17" s="37" t="n">
         <v>28.71012599578554</v>
       </c>
+      <c r="V17" s="40" t="n">
+        <v>931291.1409283208</v>
+      </c>
+      <c r="W17" s="40" t="n">
+        <v>1362542.660036802</v>
+      </c>
+      <c r="X17" s="41" t="n">
+        <v>1.463068422060372</v>
+      </c>
+      <c r="Y17" s="40" t="n">
+        <v>107685.3837162277</v>
+      </c>
+      <c r="Z17" s="40" t="n">
+        <v>70317.00532145283</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="34" t="n">
@@ -4295,6 +4865,21 @@
       <c r="U18" s="37" t="n">
         <v>25.72519634063949</v>
       </c>
+      <c r="V18" s="40" t="n">
+        <v>2177088.604877107</v>
+      </c>
+      <c r="W18" s="40" t="n">
+        <v>3963443.759269666</v>
+      </c>
+      <c r="X18" s="41" t="n">
+        <v>1.820524782680306</v>
+      </c>
+      <c r="Y18" s="40" t="n">
+        <v>301367.4532707998</v>
+      </c>
+      <c r="Z18" s="40" t="n">
+        <v>154055.1287634539</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="34" t="n">
@@ -4360,6 +4945,21 @@
       <c r="U19" s="37" t="n">
         <v>14.88463038725362</v>
       </c>
+      <c r="V19" s="40" t="n">
+        <v>1594652.173291156</v>
+      </c>
+      <c r="W19" s="40" t="n">
+        <v>1934497.265401721</v>
+      </c>
+      <c r="X19" s="41" t="n">
+        <v>1.213115498039406</v>
+      </c>
+      <c r="Y19" s="40" t="n">
+        <v>88313.55276901214</v>
+      </c>
+      <c r="Z19" s="40" t="n">
+        <v>71130.67781712321</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="34" t="n">
@@ -4424,6 +5024,21 @@
       </c>
       <c r="U20" s="37" t="n">
         <v>24.34586795511529</v>
+      </c>
+      <c r="V20" s="40" t="n">
+        <v>449214.0917825571</v>
+      </c>
+      <c r="W20" s="40" t="n">
+        <v>734469.2863935578</v>
+      </c>
+      <c r="X20" s="41" t="n">
+        <v>1.635009452795793</v>
+      </c>
+      <c r="Y20" s="40" t="n">
+        <v>62732.82268931206</v>
+      </c>
+      <c r="Z20" s="40" t="n">
+        <v>36170.3015291577</v>
       </c>
     </row>
   </sheetData>
@@ -4437,7 +5052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -4453,14 +5068,14 @@
     <row r="2">
       <c r="A2" s="44" t="inlineStr">
         <is>
-          <t>Gerada/atualizada em 15/10/2026 (modelo adotado trocado em 26/10/2026) por Scripts/gerar_planilha_comparacao.py a partir de: eventos_processados_manuais.xlsx, comparacao_volumes_medido_vs_calculado.csv,</t>
+          <t>Gerada/atualizada em 15/10/2026 (modelo adotado trocado em 26/10/2026 e de novo em 28/10/2026, para o modelo oficial) por Scripts/gerar_planilha_comparacao.py a partir de: eventos_processados_manuais.xlsx, comparacao_volumes_medido_vs_calculado.csv,</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>comparacao_qpico_convolucao_medido_vs_calculado.csv, comparacao_SY_previsao_vs_restrito.csv, comparacao_SY_modelo_com_base.csv (vazão de base, não adotado) e comparacao_SY_so_direto.csv (adotado).</t>
+          <t>comparacao_qpico_convolucao_medido_vs_calculado.csv, comparacao_SY_previsao_vs_restrito.csv, comparacao_SY_modelo_com_base.csv (vazão de base, não adotado), comparacao_SY_so_direto.csv (modelo de 26/10, não adotado) e comparacao_SY_lambda005_woodward.csv (ADOTADO, oficial de 28/10/2026).</t>
         </is>
       </c>
     </row>
@@ -4498,85 +5113,92 @@
     <row r="9">
       <c r="A9" s="44" t="inlineStr">
         <is>
-          <t>• ADOTADO (26/10/2026): só escoamento direto, sem termo de vazão de base. Calculado: Q do SCS-CN (λ = 0,20); forçado: Q reescalado para o escoamento direto medido. Compara-se com a carga TOTAL medida (todo o sedimento do evento é atribuído ao escoamento superficial).</t>
+          <t>• ADOTADO (oficial, 28/10/2026): só escoamento direto, sem termo de vazão de base. MC: Q do SCS-CN com CN-I, λ = 0,05 e S convertido (Woodward et al., 2003); MFM: Q reescalado para o escoamento direto medido. Compara-se com a carga TOTAL medida (todo o sedimento do evento é atribuído ao escoamento superficial).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="44" t="inlineStr">
         <is>
-          <t>• Nesta planilha todas as escalas c são ajustadas por mínimos quadrados lineares; no texto do TCC a calibração adotada é em log (ver TCC_Texto/tabelas/).</t>
+          <t>• Não adotado (26/10/2026): o mesmo desenho com λ = 0,20 e sem converter S.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="44" t="inlineStr">
         <is>
-          <t>• Não adotado (15 a 26/10/2026): Q = escoamento direto + lâmina de vazão de base prevista, uniforme (kb·Qb_inicio·duração). Removido: a vazão de base não produz erosão nas encostas.</t>
+          <t>• Nesta planilha todas as escalas c são ajustadas por mínimos quadrados lineares; no texto do TCC a calibração adotada é em log (ver TCC_Texto/tabelas/).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="44" t="inlineStr">
         <is>
-          <t>• Sem MUSLE: modelos triviais (SY proporcional ao volume ou à chuva), com um parâmetro c. Servem de régua: um modelo espacializado só se justifica se superar isso.</t>
+          <t>• Não adotado (15 a 26/10/2026): Q = escoamento direto + lâmina de vazão de base prevista, uniforme (kb·Qb_inicio·duração). Removido: a vazão de base não produz erosão nas encostas.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="44" t="inlineStr">
         <is>
+          <t>• Sem MUSLE: modelos triviais (SY proporcional ao volume ou à chuva), com um parâmetro c. Servem de régua: um modelo espacializado só se justifica se superar isso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="44" t="inlineStr">
+        <is>
           <t>• α e β livres e FCI/DSC são experimentos que não foram adotados (valores só in-sample).</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="44" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="43" t="inlineStr">
+      <c r="A15" s="44" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="43" t="inlineStr">
         <is>
           <t>Pontos de atenção</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="44" t="inlineStr">
-        <is>
-          <t>• T_R_m3 (volume 'medido') = soma das vazões horárias × 3600: é o volume TOTAL, inclui a vazão de base (34–55%). SYY_t é a carga total (Q·CSS). O SCS-CN calcula só escoamento direto.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="44" t="inlineStr">
         <is>
-          <t>• NSE in-sample é otimista; o leave-one-out (c, e no modelo adotado também kb, refeitos sem o evento testado) é o valor honesto. Para α/β livres e FCI/DSC não foi calculado.</t>
+          <t>• T_R_m3 (volume 'medido') = soma das vazões horárias × 3600: é o volume TOTAL, inclui a vazão de base (34–55%). SYY_t é a carga total (Q·CSS). O SCS-CN calcula só escoamento direto.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="44" t="inlineStr">
         <is>
-          <t>• O evento 15 responde por 49% da variância do SY medido; veja a coluna 'NSE sem o evento 15'. Com n = 17, os intervalos são largos (bootstrap do NSE do modelo adotado: [−0,96; 0,88]).</t>
+          <t>• NSE in-sample é otimista; o leave-one-out (c, e no modelo adotado também kb, refeitos sem o evento testado) é o valor honesto. Para α/β livres e FCI/DSC não foi calculado.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="44" t="inlineStr">
         <is>
-          <t>• 'Q forçado', 'D e qp medidos' e os modelos 'Sem MUSLE' usam dado medido do evento; não são previsões puras e não devem ser comparados diretamente com a previsão de Hao et al. (2022).</t>
+          <t>• O evento 15 responde por 49% da variância do SY medido; veja a coluna 'NSE sem o evento 15'. Com n = 17, os intervalos são largos (bootstrap do NSE do modelo de dois componentes, não adotado: [-0,96; 0,88]).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="44" t="inlineStr">
         <is>
-          <t>• No modelo adotado, a duração é a janela observada do evento, kb é ajustado nos mesmos 17 eventos e λ foi fixado em 0,20 (padrão) depois de ver diagnósticos com outros valores.</t>
+          <t>• 'Q forçado', 'D e qp medidos' e os modelos 'Sem MUSLE' usam dado medido do evento; não são previsões puras e não devem ser comparados diretamente com a previsão de Hao et al. (2022).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="44" t="inlineStr">
+        <is>
+          <t>• No modelo oficial, λ = 0,05 com S convertido e o CN-I foram escolhidos olhando os mesmos 17 eventos (ver limitações no TCC). No modelo de dois componentes (não adotado), a duração é a janela observada e kb é ajustado nos mesmos 17 eventos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="44" t="inlineStr">
         <is>
           <t>• Os valores por evento de α/β livres e de FCI/DSC vêm das saídas de calibrar_alfa_beta_pixel.py (17/09) e da recalibração com a Eq. 8 exata (02/10); o FCI/DSC está arredondado em t.</t>
         </is>

</xml_diff>